<commit_message>
feat: add script to do structure feature extraction
</commit_message>
<xml_diff>
--- a/data/proteomics/organell_protein_ratio_rosemary.xlsx
+++ b/data/proteomics/organell_protein_ratio_rosemary.xlsx
@@ -1276,22 +1276,22 @@
         <v>0.001138145322776526</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00075640249831066</v>
+        <v>0.0007564024983106602</v>
       </c>
       <c r="E2" t="n">
         <v>0.009598240105774959</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2647587701603151</v>
+        <v>0.2647587701603152</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5835637813424227</v>
+        <v>0.5835637813424233</v>
       </c>
       <c r="H2" t="n">
-        <v>0.280762087383224</v>
+        <v>0.2807620873832239</v>
       </c>
       <c r="I2" t="n">
-        <v>0.08811556074491009</v>
+        <v>0.08811556074491017</v>
       </c>
       <c r="J2" t="n">
         <v>0.02301410843838039</v>
@@ -1300,28 +1300,28 @@
         <v>0.1238652254207412</v>
       </c>
       <c r="L2" t="n">
-        <v>0.03168293346528692</v>
+        <v>0.03168293346528693</v>
       </c>
       <c r="M2" t="n">
         <v>0.004368911114365766</v>
       </c>
       <c r="N2" t="n">
-        <v>0.02187998626371159</v>
+        <v>0.02187998626371158</v>
       </c>
       <c r="O2" t="n">
-        <v>0.003299161701704413</v>
+        <v>0.003299161701704412</v>
       </c>
       <c r="P2" t="n">
-        <v>0.004943010874955365</v>
+        <v>0.004943010874955367</v>
       </c>
       <c r="Q2" t="n">
         <v>0.007299149278678302</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0064406365463601</v>
+        <v>0.006440636546360101</v>
       </c>
       <c r="S2" t="n">
-        <v>0.004349487013014682</v>
+        <v>0.004349487013014684</v>
       </c>
       <c r="T2" t="n">
         <v>0.01245148353819309</v>
@@ -1333,7 +1333,7 @@
         <v>0.001673429335754054</v>
       </c>
       <c r="W2" t="n">
-        <v>0.05663180859787956</v>
+        <v>0.05663180859787955</v>
       </c>
       <c r="X2" t="n">
         <v>0.0002561871569803065</v>
@@ -1342,28 +1342,28 @@
         <v>0.003445284789320332</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.003091116167185114</v>
+        <v>0.003091116167185115</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.02044826382745894</v>
+        <v>0.02044826382745893</v>
       </c>
       <c r="AB2" t="n">
         <v>0.0008307916238502618</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.03615553610610975</v>
+        <v>0.03615553610610973</v>
       </c>
       <c r="AD2" t="n">
-        <v>5.655671841690027e-05</v>
+        <v>5.655671841690028e-05</v>
       </c>
       <c r="AE2" t="n">
         <v>1.370749101543504e-05</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.05163401771683859</v>
+        <v>0.05163401771683861</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.03398950311822549</v>
+        <v>0.0339895031182255</v>
       </c>
       <c r="AH2" t="n">
         <v>0.001819325671496335</v>
@@ -1375,13 +1375,13 @@
         <v>0.002717652373286961</v>
       </c>
       <c r="AK2" t="n">
-        <v>0.01621749541868758</v>
+        <v>0.01621749541868757</v>
       </c>
       <c r="AL2" t="n">
         <v>0.000969098409233749</v>
       </c>
       <c r="AM2" t="n">
-        <v>0.0004082609748373422</v>
+        <v>0.0004082609748373423</v>
       </c>
       <c r="AN2" t="n">
         <v>0.0003148811135487377</v>
@@ -1396,7 +1396,7 @@
         <v>0.001237985231383709</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.006803721620284389</v>
+        <v>0.006803721620284387</v>
       </c>
       <c r="AS2" t="n">
         <v>0.0001529218598010382</v>
@@ -1405,7 +1405,7 @@
         <v>7.160717838412477e-05</v>
       </c>
       <c r="AU2" t="n">
-        <v>0.0004193415969839526</v>
+        <v>0.0004193415969839525</v>
       </c>
       <c r="AV2" t="n">
         <v>0.004496829762004332</v>
@@ -1414,10 +1414,10 @@
         <v>0.002690212388466481</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.000260692687935699</v>
+        <v>0.0002606926879356991</v>
       </c>
       <c r="AY2" t="n">
-        <v>0.02564207079487959</v>
+        <v>0.02564207079487958</v>
       </c>
       <c r="AZ2" t="n">
         <v>0.0006302258720994086</v>
@@ -1426,10 +1426,10 @@
         <v>0.00011278566634715</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.05068208213166546</v>
+        <v>0.05068208213166548</v>
       </c>
       <c r="BC2" t="n">
-        <v>0.008037157056752333</v>
+        <v>0.008037157056752332</v>
       </c>
       <c r="BD2" t="n">
         <v>0.0216249628274928</v>
@@ -1465,7 +1465,7 @@
         <v>0.001514882179045458</v>
       </c>
       <c r="BO2" t="n">
-        <v>8.122049296627732e-05</v>
+        <v>8.122049296627733e-05</v>
       </c>
       <c r="BP2" t="n">
         <v>0.0002506051290756246</v>
@@ -1474,7 +1474,7 @@
         <v>0.0004009095635308535</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.0004159423476499579</v>
+        <v>0.000415942347649958</v>
       </c>
       <c r="BS2" t="n">
         <v>0.02563426646094737</v>
@@ -1495,7 +1495,7 @@
         <v>0.002471027620689082</v>
       </c>
       <c r="BY2" t="n">
-        <v>6.626471018563797e-05</v>
+        <v>6.626471018563796e-05</v>
       </c>
       <c r="BZ2" t="n">
         <v>0.00809651840137781</v>
@@ -1513,7 +1513,7 @@
         <v>0.0001286269832270554</v>
       </c>
       <c r="CE2" t="n">
-        <v>0.004296770464568454</v>
+        <v>0.004296770464568453</v>
       </c>
       <c r="CF2" t="n">
         <v>0.0007661800678651387</v>
@@ -1525,7 +1525,7 @@
         <v>0.0004302386434430936</v>
       </c>
       <c r="CI2" t="n">
-        <v>6.059673848522341e-05</v>
+        <v>6.059673848522342e-05</v>
       </c>
       <c r="CJ2" t="n">
         <v>0.007534733357598618</v>
@@ -1540,7 +1540,7 @@
         <v>2.858461671242169e-05</v>
       </c>
       <c r="CN2" t="n">
-        <v>0.0002094064012606916</v>
+        <v>0.0002094064012606915</v>
       </c>
       <c r="CO2" t="n">
         <v>0.001531535818213803</v>
@@ -1570,7 +1570,7 @@
         <v>0.0004454556700479366</v>
       </c>
       <c r="CX2" t="n">
-        <v>0.004115811913481493</v>
+        <v>0.004115811913481494</v>
       </c>
       <c r="CY2" t="n">
         <v>0.0001169367282664049</v>
@@ -1579,7 +1579,7 @@
         <v>0.0002484235842227201</v>
       </c>
       <c r="DA2" t="n">
-        <v>0.0002839159308649933</v>
+        <v>0.0002839159308649934</v>
       </c>
       <c r="DB2" t="n">
         <v>0.0004597132695445061</v>
@@ -1597,7 +1597,7 @@
         <v>0.0004404436602171758</v>
       </c>
       <c r="DG2" t="n">
-        <v>0.006184904806043987</v>
+        <v>0.006184904806043989</v>
       </c>
       <c r="DH2" t="n">
         <v>0.0004726616705908945</v>
@@ -1624,7 +1624,7 @@
         <v>0.0007246314682725262</v>
       </c>
       <c r="DP2" t="n">
-        <v>0.07177026400670203</v>
+        <v>0.07177026400670201</v>
       </c>
       <c r="DQ2" t="n">
         <v>1.060362453724319e-05</v>
@@ -1645,7 +1645,7 @@
         <v>8.069318543692785e-05</v>
       </c>
       <c r="DW2" t="n">
-        <v>0.0002891579234470404</v>
+        <v>0.0002891579234470403</v>
       </c>
       <c r="DX2" t="n">
         <v>0.0007470332889742125</v>
@@ -1778,7 +1778,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>0.4536859217675874</v>
+        <v>0.4536859217675873</v>
       </c>
       <c r="C3" t="n">
         <v>0.001190017355736136</v>
@@ -1790,25 +1790,25 @@
         <v>0.009765240334658519</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2672907387193528</v>
+        <v>0.267290738719353</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5851790127364522</v>
+        <v>0.5851790127364529</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2726503286665412</v>
+        <v>0.2726503286665413</v>
       </c>
       <c r="I3" t="n">
-        <v>0.09036794060833292</v>
+        <v>0.09036794060833289</v>
       </c>
       <c r="J3" t="n">
-        <v>0.02245936352087539</v>
+        <v>0.02245936352087538</v>
       </c>
       <c r="K3" t="n">
         <v>0.1205266605731308</v>
       </c>
       <c r="L3" t="n">
-        <v>0.03157312306134623</v>
+        <v>0.03157312306134621</v>
       </c>
       <c r="M3" t="n">
         <v>0.004179979268314905</v>
@@ -1817,19 +1817,19 @@
         <v>0.02367136443682706</v>
       </c>
       <c r="O3" t="n">
-        <v>0.003524899145616539</v>
+        <v>0.00352489914561654</v>
       </c>
       <c r="P3" t="n">
-        <v>0.005156969452704175</v>
+        <v>0.005156969452704177</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.006422106503573297</v>
+        <v>0.006422106503573299</v>
       </c>
       <c r="R3" t="n">
         <v>0.006227037417604293</v>
       </c>
       <c r="S3" t="n">
-        <v>0.004299354733573926</v>
+        <v>0.004299354733573929</v>
       </c>
       <c r="T3" t="n">
         <v>0.01193291693481766</v>
@@ -1853,13 +1853,13 @@
         <v>0.003130223312450443</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.01935157965516326</v>
+        <v>0.01935157965516325</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.0008482564582939524</v>
+        <v>0.0008482564582939526</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.03833206522084407</v>
+        <v>0.03833206522084406</v>
       </c>
       <c r="AD3" t="n">
         <v>5.418479544510544e-05</v>
@@ -1895,13 +1895,13 @@
         <v>0.0002664835091614188</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.0005537462201997648</v>
+        <v>0.0005537462201997649</v>
       </c>
       <c r="AP3" t="n">
         <v>0.0004672320248287168</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.001198341356746271</v>
+        <v>0.00119834135674627</v>
       </c>
       <c r="AR3" t="n">
         <v>0.006463141014695298</v>
@@ -1913,7 +1913,7 @@
         <v>7.683415719273801e-05</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.0005348421243772473</v>
+        <v>0.0005348421243772474</v>
       </c>
       <c r="AV3" t="n">
         <v>0.004107042457794598</v>
@@ -1922,7 +1922,7 @@
         <v>0.002666325041698565</v>
       </c>
       <c r="AX3" t="n">
-        <v>0.000243036508133451</v>
+        <v>0.0002430365081334511</v>
       </c>
       <c r="AY3" t="n">
         <v>0.02473302936598019</v>
@@ -1940,13 +1940,13 @@
         <v>0.007728441673491691</v>
       </c>
       <c r="BD3" t="n">
-        <v>0.02115811677003062</v>
+        <v>0.02115811677003063</v>
       </c>
       <c r="BE3" t="n">
         <v>0.0004833924087487743</v>
       </c>
       <c r="BF3" t="n">
-        <v>0.0008330070072213021</v>
+        <v>0.0008330070072213022</v>
       </c>
       <c r="BG3" t="n">
         <v>0.000803026569002872</v>
@@ -1955,10 +1955,10 @@
         <v>0.01287181406900986</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.0006197372534777155</v>
+        <v>0.0006197372534777154</v>
       </c>
       <c r="BJ3" t="n">
-        <v>1.264342697978811e-05</v>
+        <v>1.264342697978812e-05</v>
       </c>
       <c r="BK3" t="n">
         <v>0.02454992913682944</v>
@@ -1967,7 +1967,7 @@
         <v>5.624979226651411e-05</v>
       </c>
       <c r="BM3" t="n">
-        <v>0.0412716072410006</v>
+        <v>0.04127160724100061</v>
       </c>
       <c r="BN3" t="n">
         <v>0.001462551414528014</v>
@@ -1979,7 +1979,7 @@
         <v>0.0002575998682265277</v>
       </c>
       <c r="BQ3" t="n">
-        <v>0.0003689030018054226</v>
+        <v>0.0003689030018054227</v>
       </c>
       <c r="BR3" t="n">
         <v>0.0004661094874081806</v>
@@ -1988,7 +1988,7 @@
         <v>0.02683856183379417</v>
       </c>
       <c r="BT3" t="n">
-        <v>0.005205724415336601</v>
+        <v>0.0052057244153366</v>
       </c>
       <c r="BU3" t="n">
         <v>0.00375616535301888</v>
@@ -2012,7 +2012,7 @@
         <v>0.0001324388756764031</v>
       </c>
       <c r="CB3" t="n">
-        <v>0.0002596116406838069</v>
+        <v>0.000259611640683807</v>
       </c>
       <c r="CC3" t="n">
         <v>0.0001492136711217892</v>
@@ -2036,10 +2036,10 @@
         <v>5.981299816791831e-05</v>
       </c>
       <c r="CJ3" t="n">
-        <v>0.007720746186446582</v>
+        <v>0.00772074618644658</v>
       </c>
       <c r="CK3" t="n">
-        <v>8.727305418555209e-06</v>
+        <v>8.727305418555207e-06</v>
       </c>
       <c r="CL3" t="n">
         <v>0.0004486990294781685</v>
@@ -2048,13 +2048,13 @@
         <v>2.658435963637779e-05</v>
       </c>
       <c r="CN3" t="n">
-        <v>0.0002064370694548269</v>
+        <v>0.0002064370694548268</v>
       </c>
       <c r="CO3" t="n">
         <v>0.001442538034624295</v>
       </c>
       <c r="CP3" t="n">
-        <v>0.001104545556367649</v>
+        <v>0.00110454555636765</v>
       </c>
       <c r="CQ3" t="n">
         <v>0.001135010553992822</v>
@@ -2063,13 +2063,13 @@
         <v>0.0004250304910871536</v>
       </c>
       <c r="CS3" t="n">
-        <v>7.708486578627711e-05</v>
+        <v>7.70848657862771e-05</v>
       </c>
       <c r="CT3" t="n">
         <v>0.0001635017911214542</v>
       </c>
       <c r="CU3" t="n">
-        <v>7.209128241335163e-05</v>
+        <v>7.209128241335161e-05</v>
       </c>
       <c r="CV3" t="n">
         <v>0.000360829288433987</v>
@@ -2078,7 +2078,7 @@
         <v>0.0004812388623252395</v>
       </c>
       <c r="CX3" t="n">
-        <v>0.003900378018905863</v>
+        <v>0.003900378018905862</v>
       </c>
       <c r="CY3" t="n">
         <v>0.000124126258843698</v>
@@ -2093,7 +2093,7 @@
         <v>0.0004780552672017843</v>
       </c>
       <c r="DC3" t="n">
-        <v>9.88962309093617e-05</v>
+        <v>9.88962309093616e-05</v>
       </c>
       <c r="DD3" t="n">
         <v>0.001378170334893687</v>
@@ -2117,10 +2117,10 @@
         <v>5.387454541560061e-05</v>
       </c>
       <c r="DK3" t="n">
-        <v>0.0009699797078465398</v>
+        <v>0.0009699797078465408</v>
       </c>
       <c r="DL3" t="n">
-        <v>0.0002934917652170636</v>
+        <v>0.0002934917652170637</v>
       </c>
       <c r="DM3" t="n">
         <v>0.0001251137037567987</v>
@@ -2129,13 +2129,13 @@
         <v>2.846700890089106e-05</v>
       </c>
       <c r="DO3" t="n">
-        <v>0.0006712545820733941</v>
+        <v>0.000671254582073394</v>
       </c>
       <c r="DP3" t="n">
-        <v>0.06891074474912709</v>
+        <v>0.06891074474912706</v>
       </c>
       <c r="DQ3" t="n">
-        <v>1.06445408191453e-05</v>
+        <v>1.064454081914529e-05</v>
       </c>
       <c r="DR3" t="n">
         <v>9.566710355794177e-05</v>
@@ -2144,7 +2144,7 @@
         <v>0.003265706118986035</v>
       </c>
       <c r="DT3" t="n">
-        <v>0.001457081899758115</v>
+        <v>0.001457081899758114</v>
       </c>
       <c r="DU3" t="n">
         <v>0.003462906833552784</v>
@@ -2186,7 +2186,7 @@
         <v>5.695606790626441e-05</v>
       </c>
       <c r="EH3" t="n">
-        <v>3.534571896786013e-05</v>
+        <v>3.534571896786012e-05</v>
       </c>
       <c r="EI3" t="n">
         <v>2.550314938926626e-05</v>
@@ -2298,16 +2298,16 @@
         <v>0.009531187683197603</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2704048328691838</v>
+        <v>0.2704048328691839</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5778917462687787</v>
+        <v>0.5778917462687791</v>
       </c>
       <c r="H4" t="n">
         <v>0.255821182078385</v>
       </c>
       <c r="I4" t="n">
-        <v>0.07947888368535576</v>
+        <v>0.07947888368535574</v>
       </c>
       <c r="J4" t="n">
         <v>0.02271766915324992</v>
@@ -2322,19 +2322,19 @@
         <v>0.0041699906214876</v>
       </c>
       <c r="N4" t="n">
-        <v>0.02616070204960104</v>
+        <v>0.02616070204960105</v>
       </c>
       <c r="O4" t="n">
-        <v>0.003599261445777715</v>
+        <v>0.003599261445777716</v>
       </c>
       <c r="P4" t="n">
-        <v>0.004701502298385578</v>
+        <v>0.004701502298385577</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.006494758845649595</v>
+        <v>0.006494758845649596</v>
       </c>
       <c r="R4" t="n">
-        <v>0.00579236105791163</v>
+        <v>0.005792361057911629</v>
       </c>
       <c r="S4" t="n">
         <v>0.004266624905191249</v>
@@ -2355,19 +2355,19 @@
         <v>0.000334954037722334</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.00346652532020754</v>
+        <v>0.003466525320207539</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.00291322575477225</v>
+        <v>0.002913225754772251</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.02024379977189248</v>
+        <v>0.02024379977189249</v>
       </c>
       <c r="AB4" t="n">
         <v>0.0009228730472713821</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.03930560113956549</v>
+        <v>0.0393056011395655</v>
       </c>
       <c r="AD4" t="n">
         <v>5.802075169389524e-05</v>
@@ -2379,25 +2379,25 @@
         <v>0.06482912571748299</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.03962589797069917</v>
+        <v>0.03962589797069918</v>
       </c>
       <c r="AH4" t="n">
         <v>0.001709215079799333</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.00105532042093492</v>
+        <v>0.001055320420934921</v>
       </c>
       <c r="AJ4" t="n">
         <v>0.002642914915330515</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.01603931407200481</v>
+        <v>0.0160393140720048</v>
       </c>
       <c r="AL4" t="n">
         <v>0.001019689985894211</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.0004689816751697236</v>
+        <v>0.0004689816751697237</v>
       </c>
       <c r="AN4" t="n">
         <v>0.0002779340070911843</v>
@@ -2412,7 +2412,7 @@
         <v>0.001227862258222554</v>
       </c>
       <c r="AR4" t="n">
-        <v>0.005829649317944525</v>
+        <v>0.005829649317944527</v>
       </c>
       <c r="AS4" t="n">
         <v>0.0001438831992132121</v>
@@ -2433,7 +2433,7 @@
         <v>0.0002517308230112055</v>
       </c>
       <c r="AY4" t="n">
-        <v>0.02374874757143994</v>
+        <v>0.02374874757143995</v>
       </c>
       <c r="AZ4" t="n">
         <v>0.0006107485110117163</v>
@@ -2442,22 +2442,22 @@
         <v>0.000114261125826021</v>
       </c>
       <c r="BB4" t="n">
-        <v>0.04983176326419914</v>
+        <v>0.04983176326419915</v>
       </c>
       <c r="BC4" t="n">
-        <v>0.007896109753469776</v>
+        <v>0.007896109753469778</v>
       </c>
       <c r="BD4" t="n">
-        <v>0.02116731265853499</v>
+        <v>0.02116731265853497</v>
       </c>
       <c r="BE4" t="n">
-        <v>0.0005785731792104751</v>
+        <v>0.000578573179210475</v>
       </c>
       <c r="BF4" t="n">
         <v>0.0008181678991504555</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.0009868729972667602</v>
+        <v>0.0009868729972667609</v>
       </c>
       <c r="BH4" t="n">
         <v>0.0142493442945973</v>
@@ -2466,13 +2466,13 @@
         <v>0.0004567447713269001</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0.0002016347786902534</v>
+        <v>0.0002016347786902535</v>
       </c>
       <c r="BK4" t="n">
         <v>0.02364571808258182</v>
       </c>
       <c r="BL4" t="n">
-        <v>6.753914185495205e-05</v>
+        <v>6.753914185495207e-05</v>
       </c>
       <c r="BM4" t="n">
         <v>0.03973282024896643</v>
@@ -2481,10 +2481,10 @@
         <v>0.001450579693027305</v>
       </c>
       <c r="BO4" t="n">
-        <v>7.662702977880792e-05</v>
+        <v>7.662702977880793e-05</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.0002423757442130722</v>
+        <v>0.0002423757442130721</v>
       </c>
       <c r="BQ4" t="n">
         <v>0.0003386536608254527</v>
@@ -2514,13 +2514,13 @@
         <v>6.33521601827009e-05</v>
       </c>
       <c r="BZ4" t="n">
-        <v>0.008178217921525312</v>
+        <v>0.008178217921525311</v>
       </c>
       <c r="CA4" t="n">
-        <v>0.0001245319921969532</v>
+        <v>0.0001245319921969533</v>
       </c>
       <c r="CB4" t="n">
-        <v>0.0002517170632457235</v>
+        <v>0.0002517170632457234</v>
       </c>
       <c r="CC4" t="n">
         <v>0.000145661773098678</v>
@@ -2535,13 +2535,13 @@
         <v>0.0008787308039256302</v>
       </c>
       <c r="CG4" t="n">
-        <v>0.003170612888506208</v>
+        <v>0.003170612888506209</v>
       </c>
       <c r="CH4" t="n">
         <v>0.0004205276441955875</v>
       </c>
       <c r="CI4" t="n">
-        <v>6.446543949698327e-05</v>
+        <v>6.446543949698325e-05</v>
       </c>
       <c r="CJ4" t="n">
         <v>0.008602033057261954</v>
@@ -2571,16 +2571,16 @@
         <v>0.0004018979955411816</v>
       </c>
       <c r="CS4" t="n">
-        <v>6.657676969777369e-05</v>
+        <v>6.657676969777368e-05</v>
       </c>
       <c r="CT4" t="n">
-        <v>0.0001513424192276227</v>
+        <v>0.0001513424192276226</v>
       </c>
       <c r="CU4" t="n">
-        <v>8.859966220996153e-05</v>
+        <v>8.859966220996152e-05</v>
       </c>
       <c r="CV4" t="n">
-        <v>0.0003892256446475493</v>
+        <v>0.0003892256446475494</v>
       </c>
       <c r="CW4" t="n">
         <v>0.000429806564708727</v>
@@ -2592,16 +2592,16 @@
         <v>0.0001179787916173633</v>
       </c>
       <c r="CZ4" t="n">
-        <v>0.0002448763264696968</v>
+        <v>0.0002448763264696966</v>
       </c>
       <c r="DA4" t="n">
-        <v>0.00025241209015792</v>
+        <v>0.0002524120901579198</v>
       </c>
       <c r="DB4" t="n">
-        <v>0.0005324967557723864</v>
+        <v>0.0005324967557723867</v>
       </c>
       <c r="DC4" t="n">
-        <v>7.592779161251312e-05</v>
+        <v>7.592779161251314e-05</v>
       </c>
       <c r="DD4" t="n">
         <v>0.001386644903557045</v>
@@ -2613,13 +2613,13 @@
         <v>0.0003658479336120572</v>
       </c>
       <c r="DG4" t="n">
-        <v>0.006181245156015991</v>
+        <v>0.00618124515601599</v>
       </c>
       <c r="DH4" t="n">
-        <v>0.0005544673486470456</v>
+        <v>0.0005544673486470455</v>
       </c>
       <c r="DI4" t="n">
-        <v>7.597458918222002e-05</v>
+        <v>7.597458918222001e-05</v>
       </c>
       <c r="DJ4" t="n">
         <v>4.25350803238105e-05</v>
@@ -2628,7 +2628,7 @@
         <v>0.0009519100974202362</v>
       </c>
       <c r="DL4" t="n">
-        <v>0.0002972217646922551</v>
+        <v>0.0002972217646922552</v>
       </c>
       <c r="DM4" t="n">
         <v>0.0001183785616395543</v>
@@ -2637,10 +2637,10 @@
         <v>2.392159993273484e-05</v>
       </c>
       <c r="DO4" t="n">
-        <v>0.0007119959987661356</v>
+        <v>0.0007119959987661359</v>
       </c>
       <c r="DP4" t="n">
-        <v>0.07038673500289598</v>
+        <v>0.07038673500289599</v>
       </c>
       <c r="DQ4" t="n">
         <v>1.114338984082168e-05</v>
@@ -2649,16 +2649,16 @@
         <v>8.88409976803437e-05</v>
       </c>
       <c r="DS4" t="n">
-        <v>0.003242113559274936</v>
+        <v>0.003242113559274935</v>
       </c>
       <c r="DT4" t="n">
         <v>0.001443633501436199</v>
       </c>
       <c r="DU4" t="n">
-        <v>0.00305973484592015</v>
+        <v>0.003059734845920151</v>
       </c>
       <c r="DV4" t="n">
-        <v>6.408431369588346e-05</v>
+        <v>6.408431369588347e-05</v>
       </c>
       <c r="DW4" t="n">
         <v>0.0002374235572865494</v>
@@ -2685,13 +2685,13 @@
         <v>1.128021600501435e-05</v>
       </c>
       <c r="EE4" t="n">
-        <v>8.989315256237304e-05</v>
+        <v>8.989315256237303e-05</v>
       </c>
       <c r="EF4" t="n">
         <v>4.209032238781583e-06</v>
       </c>
       <c r="EG4" t="n">
-        <v>6.966171439874387e-05</v>
+        <v>6.966171439874388e-05</v>
       </c>
       <c r="EH4" t="n">
         <v>2.676649847454218e-05</v>
@@ -2794,25 +2794,25 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>0.4263936587167928</v>
+        <v>0.4263936587167934</v>
       </c>
       <c r="C5" t="n">
         <v>0.001086987898536733</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0008835042779916193</v>
+        <v>0.0008835042779916192</v>
       </c>
       <c r="E5" t="n">
         <v>0.01145152515317253</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2510756159658741</v>
+        <v>0.2510756159658738</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5663175038609508</v>
+        <v>0.5663175038609521</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2676788059523421</v>
+        <v>0.2676788059523418</v>
       </c>
       <c r="I5" t="n">
         <v>0.08267061513837012</v>
@@ -2824,7 +2824,7 @@
         <v>0.1063878023397976</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0329607619698535</v>
+        <v>0.03296076196985351</v>
       </c>
       <c r="M5" t="n">
         <v>0.005103602078365277</v>
@@ -2839,10 +2839,10 @@
         <v>0.00589582029116055</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.007365026049752811</v>
+        <v>0.007365026049752815</v>
       </c>
       <c r="R5" t="n">
-        <v>0.00654916253638194</v>
+        <v>0.006549162536381938</v>
       </c>
       <c r="S5" t="n">
         <v>0.005024181085500312</v>
@@ -2857,22 +2857,22 @@
         <v>0.001818364429166239</v>
       </c>
       <c r="W5" t="n">
-        <v>0.04569397711134843</v>
+        <v>0.04569397711134841</v>
       </c>
       <c r="X5" t="n">
-        <v>0.0003464340458299951</v>
+        <v>0.000346434045829995</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.003709320322272921</v>
+        <v>0.003709320322272919</v>
       </c>
       <c r="Z5" t="n">
         <v>0.003775004523656916</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.02314008062746433</v>
+        <v>0.02314008062746435</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.0009489254109138447</v>
+        <v>0.0009489254109138448</v>
       </c>
       <c r="AC5" t="n">
         <v>0.03725046939883496</v>
@@ -2884,7 +2884,7 @@
         <v>1.50342817885009e-05</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.05533502255064026</v>
+        <v>0.05533502255064027</v>
       </c>
       <c r="AG5" t="n">
         <v>0.03951862230956376</v>
@@ -2896,13 +2896,13 @@
         <v>0.001142437232772119</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.002926093992258347</v>
+        <v>0.002926093992258348</v>
       </c>
       <c r="AK5" t="n">
         <v>0.01661330218879135</v>
       </c>
       <c r="AL5" t="n">
-        <v>0.0009959285386042711</v>
+        <v>0.0009959285386042709</v>
       </c>
       <c r="AM5" t="n">
         <v>0.0004505326355780037</v>
@@ -2920,16 +2920,16 @@
         <v>0.001368009506652417</v>
       </c>
       <c r="AR5" t="n">
-        <v>0.006777427524272307</v>
+        <v>0.006777427524272306</v>
       </c>
       <c r="AS5" t="n">
-        <v>0.0001529538731269048</v>
+        <v>0.0001529538731269049</v>
       </c>
       <c r="AT5" t="n">
         <v>8.305051973989205e-05</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.0004347594291988384</v>
+        <v>0.0004347594291988383</v>
       </c>
       <c r="AV5" t="n">
         <v>0.00346035931239486</v>
@@ -2941,7 +2941,7 @@
         <v>0.0002546016405701657</v>
       </c>
       <c r="AY5" t="n">
-        <v>0.02786407035277116</v>
+        <v>0.02786407035277117</v>
       </c>
       <c r="AZ5" t="n">
         <v>0.0007123157257704512</v>
@@ -2950,31 +2950,31 @@
         <v>0.0001130125046276351</v>
       </c>
       <c r="BB5" t="n">
-        <v>0.04316816359047597</v>
+        <v>0.04316816359047596</v>
       </c>
       <c r="BC5" t="n">
         <v>0.009081159626295385</v>
       </c>
       <c r="BD5" t="n">
-        <v>0.02833203554007147</v>
+        <v>0.02833203554007145</v>
       </c>
       <c r="BE5" t="n">
         <v>0.0005431514543861904</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.0009011511308431917</v>
+        <v>0.0009011511308431915</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.0008672758183233374</v>
+        <v>0.0008672758183233375</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.01886638236493762</v>
+        <v>0.01886638236493761</v>
       </c>
       <c r="BI5" t="n">
         <v>0.000532002414147426</v>
       </c>
       <c r="BJ5" t="n">
-        <v>5.66409514733609e-06</v>
+        <v>5.664095147336091e-06</v>
       </c>
       <c r="BK5" t="n">
         <v>0.01865760314305323</v>
@@ -2989,7 +2989,7 @@
         <v>0.001551270622380146</v>
       </c>
       <c r="BO5" t="n">
-        <v>8.051745426837371e-05</v>
+        <v>8.051745426837372e-05</v>
       </c>
       <c r="BP5" t="n">
         <v>0.0002739858649026024</v>
@@ -3007,19 +3007,19 @@
         <v>0.005515556241707839</v>
       </c>
       <c r="BU5" t="n">
-        <v>0.003766606529781044</v>
+        <v>0.003766606529781043</v>
       </c>
       <c r="BV5" t="n">
-        <v>0.003386697658783602</v>
+        <v>0.003386697658783601</v>
       </c>
       <c r="BW5" t="n">
         <v>1.076583434027208e-05</v>
       </c>
       <c r="BX5" t="n">
-        <v>0.002528397896113922</v>
+        <v>0.002528397896113923</v>
       </c>
       <c r="BY5" t="n">
-        <v>8.651104004021183e-05</v>
+        <v>8.651104004021184e-05</v>
       </c>
       <c r="BZ5" t="n">
         <v>0.009512952866026598</v>
@@ -3058,10 +3058,10 @@
         <v>1.013994484564103e-05</v>
       </c>
       <c r="CL5" t="n">
-        <v>0.0005073825807525251</v>
+        <v>0.0005073825807525252</v>
       </c>
       <c r="CM5" t="n">
-        <v>2.858312715415653e-05</v>
+        <v>2.858312715415652e-05</v>
       </c>
       <c r="CN5" t="n">
         <v>0.0002176112779424776</v>
@@ -3070,7 +3070,7 @@
         <v>0.001279569521459332</v>
       </c>
       <c r="CP5" t="n">
-        <v>0.0008902051093832292</v>
+        <v>0.0008902051093832294</v>
       </c>
       <c r="CQ5" t="n">
         <v>0.001117470662754544</v>
@@ -3079,7 +3079,7 @@
         <v>0.0004787372356143592</v>
       </c>
       <c r="CS5" t="n">
-        <v>8.268069879698985e-05</v>
+        <v>8.268069879698987e-05</v>
       </c>
       <c r="CT5" t="n">
         <v>0.0001997205532182193</v>
@@ -3088,7 +3088,7 @@
         <v>0.0001015853022629581</v>
       </c>
       <c r="CV5" t="n">
-        <v>0.0003864954127770404</v>
+        <v>0.0003864954127770403</v>
       </c>
       <c r="CW5" t="n">
         <v>0.0004041246547790937</v>
@@ -3112,7 +3112,7 @@
         <v>0.0001199288122377834</v>
       </c>
       <c r="DD5" t="n">
-        <v>0.001495316833425644</v>
+        <v>0.001495316833425643</v>
       </c>
       <c r="DE5" t="n">
         <v>9.034826622501904e-06</v>
@@ -3121,13 +3121,13 @@
         <v>0.0004459959125028116</v>
       </c>
       <c r="DG5" t="n">
-        <v>0.006131116771282704</v>
+        <v>0.006131116771282706</v>
       </c>
       <c r="DH5" t="n">
         <v>0.0005141827829695761</v>
       </c>
       <c r="DI5" t="n">
-        <v>8.205786339171998e-05</v>
+        <v>8.205786339171997e-05</v>
       </c>
       <c r="DJ5" t="n">
         <v>5.70685716540379e-05</v>
@@ -3145,7 +3145,7 @@
         <v>3.365077072887017e-05</v>
       </c>
       <c r="DO5" t="n">
-        <v>0.0009604147927331547</v>
+        <v>0.0009604147927331548</v>
       </c>
       <c r="DP5" t="n">
         <v>0.07920413304493257</v>
@@ -3172,7 +3172,7 @@
         <v>0.0003461417547028038</v>
       </c>
       <c r="DX5" t="n">
-        <v>0.0007990926380037985</v>
+        <v>0.0007990926380037986</v>
       </c>
       <c r="DY5" t="n">
         <v>0.000233705076129715</v>
@@ -3181,10 +3181,10 @@
         <v>0.0001993502567594431</v>
       </c>
       <c r="EA5" t="n">
-        <v>0.0004205601129810139</v>
+        <v>0.000420560112981014</v>
       </c>
       <c r="EB5" t="n">
-        <v>0.0002580396522472382</v>
+        <v>0.0002580396522472383</v>
       </c>
       <c r="EC5" t="n">
         <v>0.005365205032086626</v>
@@ -3202,10 +3202,10 @@
         <v>9.835533551432516e-05</v>
       </c>
       <c r="EH5" t="n">
-        <v>4.08143447097147e-05</v>
+        <v>4.081434470971469e-05</v>
       </c>
       <c r="EI5" t="n">
-        <v>2.837847993465129e-05</v>
+        <v>2.837847993465128e-05</v>
       </c>
       <c r="EJ5" t="n">
         <v>4.280733588173251e-05</v>
@@ -3302,28 +3302,28 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>0.4227352516911568</v>
+        <v>0.4227352516911567</v>
       </c>
       <c r="C6" t="n">
         <v>0.001066704132296637</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0008726615853132888</v>
+        <v>0.0008726615853132886</v>
       </c>
       <c r="E6" t="n">
         <v>0.01111363487178603</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2515811101390258</v>
+        <v>0.251581110139026</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5663702387268805</v>
+        <v>0.5663702387268803</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2614041969077068</v>
+        <v>0.2614041969077065</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0825767104522898</v>
+        <v>0.08257671045228983</v>
       </c>
       <c r="J6" t="n">
         <v>0.02815547285160128</v>
@@ -3332,10 +3332,10 @@
         <v>0.103011272284949</v>
       </c>
       <c r="L6" t="n">
-        <v>0.03438301543595158</v>
+        <v>0.0343830154359516</v>
       </c>
       <c r="M6" t="n">
-        <v>0.005601051590717518</v>
+        <v>0.005601051590717519</v>
       </c>
       <c r="N6" t="n">
         <v>0.02206054957389998</v>
@@ -3344,13 +3344,13 @@
         <v>0.003474109133720714</v>
       </c>
       <c r="P6" t="n">
-        <v>0.005688818709110314</v>
+        <v>0.005688818709110313</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.008061015446207555</v>
+        <v>0.008061015446207557</v>
       </c>
       <c r="R6" t="n">
-        <v>0.006791665756680056</v>
+        <v>0.006791665756680057</v>
       </c>
       <c r="S6" t="n">
         <v>0.004924852278047216</v>
@@ -3374,37 +3374,37 @@
         <v>0.003793012992107939</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.003594781959460518</v>
+        <v>0.003594781959460517</v>
       </c>
       <c r="AA6" t="n">
         <v>0.02207652046551524</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.0009343019799458824</v>
+        <v>0.0009343019799458825</v>
       </c>
       <c r="AC6" t="n">
         <v>0.04069959670922148</v>
       </c>
       <c r="AD6" t="n">
-        <v>6.224528430332484e-05</v>
+        <v>6.224528430332483e-05</v>
       </c>
       <c r="AE6" t="n">
         <v>1.352337795305108e-05</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.05545774376379076</v>
+        <v>0.05545774376379077</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.03869845786108607</v>
+        <v>0.03869845786108608</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.001821636454842894</v>
+        <v>0.001821636454842895</v>
       </c>
       <c r="AI6" t="n">
         <v>0.001109019574415851</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.002808019728542689</v>
+        <v>0.002808019728542688</v>
       </c>
       <c r="AK6" t="n">
         <v>0.01661091608057941</v>
@@ -3422,13 +3422,13 @@
         <v>0.0006060281983793638</v>
       </c>
       <c r="AP6" t="n">
-        <v>0.0005263893586533079</v>
+        <v>0.0005263893586533082</v>
       </c>
       <c r="AQ6" t="n">
         <v>0.001415472210854034</v>
       </c>
       <c r="AR6" t="n">
-        <v>0.006985426191517972</v>
+        <v>0.006985426191517971</v>
       </c>
       <c r="AS6" t="n">
         <v>0.0001425997639309064</v>
@@ -3449,7 +3449,7 @@
         <v>0.0002550161853322615</v>
       </c>
       <c r="AY6" t="n">
-        <v>0.02627862706672283</v>
+        <v>0.02627862706672282</v>
       </c>
       <c r="AZ6" t="n">
         <v>0.0007139173525756071</v>
@@ -3458,7 +3458,7 @@
         <v>0.0001118038964318673</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.04688263262378842</v>
+        <v>0.0468826326237884</v>
       </c>
       <c r="BC6" t="n">
         <v>0.009107309064640239</v>
@@ -3470,7 +3470,7 @@
         <v>0.000548128291267283</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.0009330877553775716</v>
+        <v>0.0009330877553775713</v>
       </c>
       <c r="BG6" t="n">
         <v>0.0011245813849962</v>
@@ -3485,16 +3485,16 @@
         <v>0.0002313847828477033</v>
       </c>
       <c r="BK6" t="n">
-        <v>0.0219041196173692</v>
+        <v>0.02190411961736921</v>
       </c>
       <c r="BL6" t="n">
-        <v>7.576919944009851e-05</v>
+        <v>7.57691994400985e-05</v>
       </c>
       <c r="BM6" t="n">
         <v>0.02603943026841241</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.00161356607264513</v>
+        <v>0.001613566072645129</v>
       </c>
       <c r="BO6" t="n">
         <v>8.177430860095533e-05</v>
@@ -3515,7 +3515,7 @@
         <v>0.005121530463081878</v>
       </c>
       <c r="BU6" t="n">
-        <v>0.003769445650886081</v>
+        <v>0.003769445650886079</v>
       </c>
       <c r="BV6" t="n">
         <v>0.003337774494566181</v>
@@ -3524,7 +3524,7 @@
         <v>1.054412450191566e-05</v>
       </c>
       <c r="BX6" t="n">
-        <v>0.002395879143432657</v>
+        <v>0.002395879143432656</v>
       </c>
       <c r="BY6" t="n">
         <v>8.716267927988565e-05</v>
@@ -3551,7 +3551,7 @@
         <v>0.0009932124789159391</v>
       </c>
       <c r="CG6" t="n">
-        <v>0.004416257370812519</v>
+        <v>0.00441625737081252</v>
       </c>
       <c r="CH6" t="n">
         <v>0.0004516806323105955</v>
@@ -3560,7 +3560,7 @@
         <v>4.971801122583898e-05</v>
       </c>
       <c r="CJ6" t="n">
-        <v>0.009546984340395047</v>
+        <v>0.009546984340395049</v>
       </c>
       <c r="CK6" t="n">
         <v>1.090205390824516e-05</v>
@@ -3587,7 +3587,7 @@
         <v>0.000509320767969408</v>
       </c>
       <c r="CS6" t="n">
-        <v>8.262680603546192e-05</v>
+        <v>8.26268060354619e-05</v>
       </c>
       <c r="CT6" t="n">
         <v>0.0001831861232492419</v>
@@ -3596,13 +3596,13 @@
         <v>9.85630996684478e-05</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.0003632450680907215</v>
+        <v>0.0003632450680907216</v>
       </c>
       <c r="CW6" t="n">
-        <v>0.0004555790365386943</v>
+        <v>0.0004555790365386942</v>
       </c>
       <c r="CX6" t="n">
-        <v>0.003694441908169486</v>
+        <v>0.003694441908169485</v>
       </c>
       <c r="CY6" t="n">
         <v>0.0001212824903189612</v>
@@ -3611,7 +3611,7 @@
         <v>0.0002833889747667166</v>
       </c>
       <c r="DA6" t="n">
-        <v>0.0002912877747387426</v>
+        <v>0.0002912877747387425</v>
       </c>
       <c r="DB6" t="n">
         <v>0.0005351462774161597</v>
@@ -3623,19 +3623,19 @@
         <v>0.001480312618808335</v>
       </c>
       <c r="DE6" t="n">
-        <v>9.4578980177534e-06</v>
+        <v>9.457898017753402e-06</v>
       </c>
       <c r="DF6" t="n">
         <v>0.000483594658682301</v>
       </c>
       <c r="DG6" t="n">
-        <v>0.00621338702724572</v>
+        <v>0.006213387027245721</v>
       </c>
       <c r="DH6" t="n">
-        <v>0.0005163818081614936</v>
+        <v>0.0005163818081614935</v>
       </c>
       <c r="DI6" t="n">
-        <v>7.67157452725074e-05</v>
+        <v>7.671574527250739e-05</v>
       </c>
       <c r="DJ6" t="n">
         <v>5.166602281082181e-05</v>
@@ -3644,25 +3644,25 @@
         <v>0.001064257804534139</v>
       </c>
       <c r="DL6" t="n">
-        <v>0.0003189893933449248</v>
+        <v>0.0003189893933449249</v>
       </c>
       <c r="DM6" t="n">
-        <v>0.0001161518803692998</v>
+        <v>0.0001161518803692997</v>
       </c>
       <c r="DN6" t="n">
         <v>3.071635165533999e-05</v>
       </c>
       <c r="DO6" t="n">
-        <v>0.0009615572421100846</v>
+        <v>0.0009615572421100845</v>
       </c>
       <c r="DP6" t="n">
-        <v>0.07581372615487006</v>
+        <v>0.07581372615487005</v>
       </c>
       <c r="DQ6" t="n">
         <v>1.034858085341082e-05</v>
       </c>
       <c r="DR6" t="n">
-        <v>9.938606093281591e-05</v>
+        <v>9.938606093281589e-05</v>
       </c>
       <c r="DS6" t="n">
         <v>0.003129998497811821</v>
@@ -3671,7 +3671,7 @@
         <v>0.001772297936858553</v>
       </c>
       <c r="DU6" t="n">
-        <v>0.003615452291658845</v>
+        <v>0.003615452291658844</v>
       </c>
       <c r="DV6" t="n">
         <v>8.571568568734518e-05</v>
@@ -3683,7 +3683,7 @@
         <v>0.0008145095895362592</v>
       </c>
       <c r="DY6" t="n">
-        <v>0.0002220324034119362</v>
+        <v>0.0002220324034119361</v>
       </c>
       <c r="DZ6" t="n">
         <v>0.0001935972120078755</v>
@@ -3704,10 +3704,10 @@
         <v>8.012324544205515e-05</v>
       </c>
       <c r="EF6" t="n">
-        <v>4.91584776143842e-06</v>
+        <v>4.915847761438418e-06</v>
       </c>
       <c r="EG6" t="n">
-        <v>9.491487454593311e-05</v>
+        <v>9.491487454593313e-05</v>
       </c>
       <c r="EH6" t="n">
         <v>4.020648351617218e-05</v>
@@ -3810,13 +3810,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.4512088687422484</v>
+        <v>0.4512088687422486</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0007296455465054329</v>
+        <v>0.000729645546505433</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0006821625563865078</v>
+        <v>0.0006821625563865077</v>
       </c>
       <c r="E7" t="n">
         <v>0.01116522728610826</v>
@@ -3825,7 +3825,7 @@
         <v>0.2574374059033812</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5881230487205839</v>
+        <v>0.5881230487205847</v>
       </c>
       <c r="H7" t="n">
         <v>0.3024792976751285</v>
@@ -3837,10 +3837,10 @@
         <v>0.02335995527047988</v>
       </c>
       <c r="K7" t="n">
-        <v>0.141051231127172</v>
+        <v>0.1410512311271719</v>
       </c>
       <c r="L7" t="n">
-        <v>0.02573062721388294</v>
+        <v>0.02573062721388295</v>
       </c>
       <c r="M7" t="n">
         <v>0.00321457763481158</v>
@@ -3849,19 +3849,19 @@
         <v>0.0209946720768532</v>
       </c>
       <c r="O7" t="n">
-        <v>0.005505219917798486</v>
+        <v>0.005505219917798487</v>
       </c>
       <c r="P7" t="n">
-        <v>0.003699955521931143</v>
+        <v>0.003699955521931142</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.005330180751681559</v>
+        <v>0.00533018075168156</v>
       </c>
       <c r="R7" t="n">
-        <v>0.004714260085010937</v>
+        <v>0.004714260085010939</v>
       </c>
       <c r="S7" t="n">
-        <v>0.003910361819797149</v>
+        <v>0.003910361819797151</v>
       </c>
       <c r="T7" t="n">
         <v>0.01388764138730868</v>
@@ -3876,7 +3876,7 @@
         <v>0.07958488400974721</v>
       </c>
       <c r="X7" t="n">
-        <v>0.0003261793016035721</v>
+        <v>0.0003261793016035722</v>
       </c>
       <c r="Y7" t="n">
         <v>0.004013082790983339</v>
@@ -3885,22 +3885,22 @@
         <v>0.002244172093713539</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.02289387107701319</v>
+        <v>0.02289387107701318</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.0006848128999392874</v>
+        <v>0.0006848128999392873</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.02594043055284688</v>
+        <v>0.02594043055284687</v>
       </c>
       <c r="AD7" t="n">
         <v>4.884138244872699e-05</v>
       </c>
       <c r="AE7" t="n">
-        <v>1.110510761988633e-05</v>
+        <v>1.110510761988632e-05</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.05922247508711111</v>
+        <v>0.05922247508711113</v>
       </c>
       <c r="AG7" t="n">
         <v>0.03584183200582444</v>
@@ -3918,16 +3918,16 @@
         <v>0.01932080771260236</v>
       </c>
       <c r="AL7" t="n">
-        <v>0.0006969837275471068</v>
+        <v>0.0006969837275471071</v>
       </c>
       <c r="AM7" t="n">
-        <v>0.0003128133575532775</v>
+        <v>0.0003128133575532776</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.0002579357859064338</v>
+        <v>0.0002579357859064336</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.000740839081271194</v>
+        <v>0.0007408390812711942</v>
       </c>
       <c r="AP7" t="n">
         <v>0.0005471863218728762</v>
@@ -3936,7 +3936,7 @@
         <v>0.001373412286213659</v>
       </c>
       <c r="AR7" t="n">
-        <v>0.00538689377352201</v>
+        <v>0.005386893773522009</v>
       </c>
       <c r="AS7" t="n">
         <v>0.0001172817929353189</v>
@@ -3957,7 +3957,7 @@
         <v>0.0002416101699192542</v>
       </c>
       <c r="AY7" t="n">
-        <v>0.02679733946509781</v>
+        <v>0.0267973394650978</v>
       </c>
       <c r="AZ7" t="n">
         <v>0.0006728257790560733</v>
@@ -3969,7 +3969,7 @@
         <v>0.04173120507133175</v>
       </c>
       <c r="BC7" t="n">
-        <v>0.009600289791425442</v>
+        <v>0.009600289791425451</v>
       </c>
       <c r="BD7" t="n">
         <v>0.02179742698384157</v>
@@ -4020,13 +4020,13 @@
         <v>0.02432615682297292</v>
       </c>
       <c r="BT7" t="n">
-        <v>0.00430615389297866</v>
+        <v>0.004306153892978661</v>
       </c>
       <c r="BU7" t="n">
-        <v>0.003628611241928438</v>
+        <v>0.003628611241928436</v>
       </c>
       <c r="BV7" t="n">
-        <v>0.004199792804089682</v>
+        <v>0.004199792804089681</v>
       </c>
       <c r="BW7" t="n">
         <v>1.087431983260142e-05</v>
@@ -4035,7 +4035,7 @@
         <v>0.001632798725366956</v>
       </c>
       <c r="BY7" t="n">
-        <v>5.588807925798736e-05</v>
+        <v>5.588807925798735e-05</v>
       </c>
       <c r="BZ7" t="n">
         <v>0.005234130413610691</v>
@@ -4053,7 +4053,7 @@
         <v>0.0001353063131675198</v>
       </c>
       <c r="CE7" t="n">
-        <v>0.006852712116312505</v>
+        <v>0.006852712116312503</v>
       </c>
       <c r="CF7" t="n">
         <v>0.001290224028284664</v>
@@ -4062,7 +4062,7 @@
         <v>0.002423649729756264</v>
       </c>
       <c r="CH7" t="n">
-        <v>0.00040088639552765</v>
+        <v>0.0004008863955276501</v>
       </c>
       <c r="CI7" t="n">
         <v>7.577190797293083e-05</v>
@@ -4074,7 +4074,7 @@
         <v>7.173158778315475e-06</v>
       </c>
       <c r="CL7" t="n">
-        <v>0.0003920728963800897</v>
+        <v>0.0003920728963800896</v>
       </c>
       <c r="CM7" t="n">
         <v>1.879690236546644e-05</v>
@@ -4089,13 +4089,13 @@
         <v>0.0004971401914702826</v>
       </c>
       <c r="CQ7" t="n">
-        <v>0.001121592929989775</v>
+        <v>0.001121592929989774</v>
       </c>
       <c r="CR7" t="n">
         <v>0.0005646133279953498</v>
       </c>
       <c r="CS7" t="n">
-        <v>5.676328476822276e-05</v>
+        <v>5.676328476822275e-05</v>
       </c>
       <c r="CT7" t="n">
         <v>0.0001685847910219153</v>
@@ -4113,7 +4113,7 @@
         <v>0.003766102357410378</v>
       </c>
       <c r="CY7" t="n">
-        <v>0.0001280700647111048</v>
+        <v>0.0001280700647111047</v>
       </c>
       <c r="CZ7" t="n">
         <v>0.0001803329831529484</v>
@@ -4137,7 +4137,7 @@
         <v>0.0003368678465904926</v>
       </c>
       <c r="DG7" t="n">
-        <v>0.005640154976530077</v>
+        <v>0.005640154976530079</v>
       </c>
       <c r="DH7" t="n">
         <v>0.0003976638085500405</v>
@@ -4146,7 +4146,7 @@
         <v>0.000100416437033503</v>
       </c>
       <c r="DJ7" t="n">
-        <v>6.711676852233648e-05</v>
+        <v>6.711676852233647e-05</v>
       </c>
       <c r="DK7" t="n">
         <v>0.0008727259950441484</v>
@@ -4161,7 +4161,7 @@
         <v>2.274274325243181e-05</v>
       </c>
       <c r="DO7" t="n">
-        <v>0.000706821198163366</v>
+        <v>0.0007068211981633659</v>
       </c>
       <c r="DP7" t="n">
         <v>0.08225486092525927</v>
@@ -4170,7 +4170,7 @@
         <v>6.750365975570304e-06</v>
       </c>
       <c r="DR7" t="n">
-        <v>5.037822988110055e-05</v>
+        <v>5.037822988110054e-05</v>
       </c>
       <c r="DS7" t="n">
         <v>0.002796812640718052</v>
@@ -4188,7 +4188,7 @@
         <v>0.0002421559554248662</v>
       </c>
       <c r="DX7" t="n">
-        <v>0.00045249441386706</v>
+        <v>0.0004524944138670601</v>
       </c>
       <c r="DY7" t="n">
         <v>0.0002223111673012861</v>
@@ -4215,7 +4215,7 @@
         <v>2.891273521419899e-06</v>
       </c>
       <c r="EG7" t="n">
-        <v>7.233880403028732e-05</v>
+        <v>7.233880403028733e-05</v>
       </c>
       <c r="EH7" t="n">
         <v>2.570755751536343e-05</v>
@@ -4318,25 +4318,25 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>0.4185874707716747</v>
+        <v>0.418587470771675</v>
       </c>
       <c r="C8" t="n">
         <v>0.0009182979219400753</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0008646926985152683</v>
+        <v>0.0008646926985152691</v>
       </c>
       <c r="E8" t="n">
         <v>0.01257891601691838</v>
       </c>
       <c r="F8" t="n">
-        <v>0.242073961629441</v>
+        <v>0.2420739616294409</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5603785905562928</v>
+        <v>0.5603785905562924</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2665094618397647</v>
+        <v>0.2665094618397649</v>
       </c>
       <c r="I8" t="n">
         <v>0.07736590648399899</v>
@@ -4348,7 +4348,7 @@
         <v>0.1094202738713886</v>
       </c>
       <c r="L8" t="n">
-        <v>0.03495570200526717</v>
+        <v>0.03495570200526718</v>
       </c>
       <c r="M8" t="n">
         <v>0.005832361432074206</v>
@@ -4366,13 +4366,13 @@
         <v>0.00856179080204846</v>
       </c>
       <c r="R8" t="n">
-        <v>0.006855887057705692</v>
+        <v>0.00685588705770569</v>
       </c>
       <c r="S8" t="n">
         <v>0.005095442367488778</v>
       </c>
       <c r="T8" t="n">
-        <v>0.01456310661122788</v>
+        <v>0.01456310661122789</v>
       </c>
       <c r="U8" t="n">
         <v>3.196061731174844e-05</v>
@@ -4381,16 +4381,16 @@
         <v>0.001826443480112324</v>
       </c>
       <c r="W8" t="n">
-        <v>0.05804575346060428</v>
+        <v>0.05804575346060426</v>
       </c>
       <c r="X8" t="n">
         <v>0.0003969114223776121</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.003705618171910458</v>
+        <v>0.003705618171910455</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.003733877196616807</v>
+        <v>0.00373387719661681</v>
       </c>
       <c r="AA8" t="n">
         <v>0.02445430028984909</v>
@@ -4399,10 +4399,10 @@
         <v>0.0008665426211706415</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.03310241668819733</v>
+        <v>0.03310241668819734</v>
       </c>
       <c r="AD8" t="n">
-        <v>4.859171621027023e-05</v>
+        <v>4.859171621027024e-05</v>
       </c>
       <c r="AE8" t="n">
         <v>1.282288369708415e-05</v>
@@ -4432,10 +4432,10 @@
         <v>0.0003989387867221434</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.0003177212584909772</v>
+        <v>0.0003177212584909771</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.0006177232733068819</v>
+        <v>0.0006177232733068818</v>
       </c>
       <c r="AP8" t="n">
         <v>0.0005141124502169301</v>
@@ -4453,7 +4453,7 @@
         <v>8.495240889889956e-05</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.0004198088393302269</v>
+        <v>0.000419808839330227</v>
       </c>
       <c r="AV8" t="n">
         <v>0.003792155694872007</v>
@@ -4465,7 +4465,7 @@
         <v>0.0002691290903528688</v>
       </c>
       <c r="AY8" t="n">
-        <v>0.03092193403290284</v>
+        <v>0.03092193403290283</v>
       </c>
       <c r="AZ8" t="n">
         <v>0.0008044312323735831</v>
@@ -4474,16 +4474,16 @@
         <v>9.961741918484205e-05</v>
       </c>
       <c r="BB8" t="n">
-        <v>0.04155325052245556</v>
+        <v>0.04155325052245559</v>
       </c>
       <c r="BC8" t="n">
-        <v>0.009546392941887702</v>
+        <v>0.009546392941887695</v>
       </c>
       <c r="BD8" t="n">
-        <v>0.03114882908089266</v>
+        <v>0.03114882908089268</v>
       </c>
       <c r="BE8" t="n">
-        <v>0.0004879574728392893</v>
+        <v>0.0004879574728392892</v>
       </c>
       <c r="BF8" t="n">
         <v>0.0008422914445381055</v>
@@ -4495,7 +4495,7 @@
         <v>0.02026350484763654</v>
       </c>
       <c r="BI8" t="n">
-        <v>0.0005591894142024214</v>
+        <v>0.0005591894142024211</v>
       </c>
       <c r="BJ8" t="n">
         <v>4.778988036757449e-06</v>
@@ -4507,10 +4507,10 @@
         <v>7.587271765914685e-05</v>
       </c>
       <c r="BM8" t="n">
-        <v>0.02704966738291014</v>
+        <v>0.02704966738291015</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.00178666884603313</v>
+        <v>0.001786668846033128</v>
       </c>
       <c r="BO8" t="n">
         <v>6.398629006414612e-05</v>
@@ -4519,28 +4519,28 @@
         <v>0.0002915317364965984</v>
       </c>
       <c r="BQ8" t="n">
-        <v>0.0005019102571873975</v>
+        <v>0.0005019102571873974</v>
       </c>
       <c r="BR8" t="n">
         <v>0.0002064377192702194</v>
       </c>
       <c r="BS8" t="n">
-        <v>0.02868939677219061</v>
+        <v>0.0286893967721906</v>
       </c>
       <c r="BT8" t="n">
-        <v>0.005601280858091069</v>
+        <v>0.005601280858091071</v>
       </c>
       <c r="BU8" t="n">
         <v>0.003942398452163197</v>
       </c>
       <c r="BV8" t="n">
-        <v>0.003728086787280035</v>
+        <v>0.003728086787280034</v>
       </c>
       <c r="BW8" t="n">
         <v>9.97568254422909e-06</v>
       </c>
       <c r="BX8" t="n">
-        <v>0.00258900389422287</v>
+        <v>0.002589003894222869</v>
       </c>
       <c r="BY8" t="n">
         <v>9.935463151683942e-05</v>
@@ -4552,7 +4552,7 @@
         <v>0.0001172876929700365</v>
       </c>
       <c r="CB8" t="n">
-        <v>0.0003382253801087038</v>
+        <v>0.0003382253801087039</v>
       </c>
       <c r="CC8" t="n">
         <v>0.000115919420787347</v>
@@ -4567,10 +4567,10 @@
         <v>0.001208180454770268</v>
       </c>
       <c r="CG8" t="n">
-        <v>0.004630124880982714</v>
+        <v>0.004630124880982715</v>
       </c>
       <c r="CH8" t="n">
-        <v>0.0004901590318621084</v>
+        <v>0.0004901590318621083</v>
       </c>
       <c r="CI8" t="n">
         <v>0.0001349790568316243</v>
@@ -4603,7 +4603,7 @@
         <v>0.0005772208703116492</v>
       </c>
       <c r="CS8" t="n">
-        <v>8.392174428003296e-05</v>
+        <v>8.392174428003303e-05</v>
       </c>
       <c r="CT8" t="n">
         <v>0.0002059257995501268</v>
@@ -4615,7 +4615,7 @@
         <v>0.0003865187223967765</v>
       </c>
       <c r="CW8" t="n">
-        <v>0.0004735773807275567</v>
+        <v>0.0004735773807275566</v>
       </c>
       <c r="CX8" t="n">
         <v>0.003969444865231082</v>
@@ -4627,10 +4627,10 @@
         <v>0.0002621734757694376</v>
       </c>
       <c r="DA8" t="n">
-        <v>0.0003016891521015849</v>
+        <v>0.000301689152101585</v>
       </c>
       <c r="DB8" t="n">
-        <v>0.0005236531152600403</v>
+        <v>0.0005236531152600402</v>
       </c>
       <c r="DC8" t="n">
         <v>0.0001135563554548111</v>
@@ -4645,7 +4645,7 @@
         <v>0.0004865141747124761</v>
       </c>
       <c r="DG8" t="n">
-        <v>0.006154011982984111</v>
+        <v>0.00615401198298411</v>
       </c>
       <c r="DH8" t="n">
         <v>0.0004619320225859645</v>
@@ -4654,13 +4654,13 @@
         <v>8.837917000834815e-05</v>
       </c>
       <c r="DJ8" t="n">
-        <v>5.505224729798112e-05</v>
+        <v>5.505224729798111e-05</v>
       </c>
       <c r="DK8" t="n">
         <v>0.001104272551395457</v>
       </c>
       <c r="DL8" t="n">
-        <v>0.0002905561949696736</v>
+        <v>0.0002905561949696735</v>
       </c>
       <c r="DM8" t="n">
         <v>0.0002104684940903178</v>
@@ -4669,19 +4669,19 @@
         <v>3.58798571110611e-05</v>
       </c>
       <c r="DO8" t="n">
-        <v>0.001105469475121426</v>
+        <v>0.001105469475121425</v>
       </c>
       <c r="DP8" t="n">
         <v>0.08960722933550004</v>
       </c>
       <c r="DQ8" t="n">
-        <v>7.635395976985975e-06</v>
+        <v>7.635395976985982e-06</v>
       </c>
       <c r="DR8" t="n">
         <v>8.461491645797574e-05</v>
       </c>
       <c r="DS8" t="n">
-        <v>0.003316283066055466</v>
+        <v>0.003316283066055467</v>
       </c>
       <c r="DT8" t="n">
         <v>0.001466811591181674</v>
@@ -4838,16 +4838,16 @@
         <v>0.01247913185216071</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2471561411295326</v>
+        <v>0.2471561411295322</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5584154370198481</v>
+        <v>0.5584154370198479</v>
       </c>
       <c r="H9" t="n">
         <v>0.2701226509151341</v>
       </c>
       <c r="I9" t="n">
-        <v>0.07900965566410828</v>
+        <v>0.07900965566410827</v>
       </c>
       <c r="J9" t="n">
         <v>0.03086140033662638</v>
@@ -4856,31 +4856,31 @@
         <v>0.1099627838772212</v>
       </c>
       <c r="L9" t="n">
-        <v>0.03457142741800375</v>
+        <v>0.03457142741800374</v>
       </c>
       <c r="M9" t="n">
         <v>0.005481639076710339</v>
       </c>
       <c r="N9" t="n">
-        <v>0.02218574555128188</v>
+        <v>0.0221857455512819</v>
       </c>
       <c r="O9" t="n">
         <v>0.005074721046069027</v>
       </c>
       <c r="P9" t="n">
-        <v>0.005538328073384968</v>
+        <v>0.005538328073384967</v>
       </c>
       <c r="Q9" t="n">
         <v>0.008178306797290615</v>
       </c>
       <c r="R9" t="n">
-        <v>0.006605363965043273</v>
+        <v>0.006605363965043275</v>
       </c>
       <c r="S9" t="n">
         <v>0.005230095749707733</v>
       </c>
       <c r="T9" t="n">
-        <v>0.01465627153899894</v>
+        <v>0.01465627153899893</v>
       </c>
       <c r="U9" t="n">
         <v>3.208849545458228e-05</v>
@@ -4889,7 +4889,7 @@
         <v>0.001902801944076172</v>
       </c>
       <c r="W9" t="n">
-        <v>0.05663733234435009</v>
+        <v>0.05663733234435007</v>
       </c>
       <c r="X9" t="n">
         <v>0.0003867427853699841</v>
@@ -4898,7 +4898,7 @@
         <v>0.003764931573672967</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.003550377360484212</v>
+        <v>0.003550377360484213</v>
       </c>
       <c r="AA9" t="n">
         <v>0.02430260618052312</v>
@@ -4907,7 +4907,7 @@
         <v>0.0008675842159623827</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.03285569065337129</v>
+        <v>0.03285569065337128</v>
       </c>
       <c r="AD9" t="n">
         <v>5.171796060828524e-05</v>
@@ -4916,10 +4916,10 @@
         <v>1.354079471067649e-05</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.05533985609095332</v>
+        <v>0.05533985609095333</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.03841670912756601</v>
+        <v>0.038416709127566</v>
       </c>
       <c r="AH9" t="n">
         <v>0.002034546116294713</v>
@@ -4928,7 +4928,7 @@
         <v>0.001357246287497028</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.002919035942770773</v>
+        <v>0.002919035942770774</v>
       </c>
       <c r="AK9" t="n">
         <v>0.02009532077634887</v>
@@ -4964,13 +4964,13 @@
         <v>0.0004064401179867325</v>
       </c>
       <c r="AV9" t="n">
-        <v>0.003700794729834849</v>
+        <v>0.00370079472983485</v>
       </c>
       <c r="AW9" t="n">
         <v>0.003839133010820785</v>
       </c>
       <c r="AX9" t="n">
-        <v>0.0002821960810717486</v>
+        <v>0.0002821960810717487</v>
       </c>
       <c r="AY9" t="n">
         <v>0.03069738614254761</v>
@@ -4982,13 +4982,13 @@
         <v>9.464275449122237e-05</v>
       </c>
       <c r="BB9" t="n">
-        <v>0.03927097684150835</v>
+        <v>0.03927097684150833</v>
       </c>
       <c r="BC9" t="n">
         <v>0.009638331446216694</v>
       </c>
       <c r="BD9" t="n">
-        <v>0.03080030862609277</v>
+        <v>0.03080030862609279</v>
       </c>
       <c r="BE9" t="n">
         <v>0.0005464423400826753</v>
@@ -5009,16 +5009,16 @@
         <v>0.0001984838200449529</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.01807001660112404</v>
+        <v>0.01807001660112405</v>
       </c>
       <c r="BL9" t="n">
         <v>7.746115098640577e-05</v>
       </c>
       <c r="BM9" t="n">
-        <v>0.02744036884264832</v>
+        <v>0.02744036884264833</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.001771729597464904</v>
+        <v>0.001771729597464905</v>
       </c>
       <c r="BO9" t="n">
         <v>6.284282435804147e-05</v>
@@ -5027,7 +5027,7 @@
         <v>0.0002706966659756605</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.0005046484597673816</v>
+        <v>0.0005046484597673817</v>
       </c>
       <c r="BR9" t="n">
         <v>0.0001822298882981393</v>
@@ -5036,10 +5036,10 @@
         <v>0.02901067621456172</v>
       </c>
       <c r="BT9" t="n">
-        <v>0.005379728394836999</v>
+        <v>0.005379728394837002</v>
       </c>
       <c r="BU9" t="n">
-        <v>0.003743452435176626</v>
+        <v>0.003743452435176627</v>
       </c>
       <c r="BV9" t="n">
         <v>0.003755422488185732</v>
@@ -5060,7 +5060,7 @@
         <v>0.000120020768916203</v>
       </c>
       <c r="CB9" t="n">
-        <v>0.000340501776407284</v>
+        <v>0.0003405017764072841</v>
       </c>
       <c r="CC9" t="n">
         <v>0.0001165114703230358</v>
@@ -5069,13 +5069,13 @@
         <v>0.0001772445490583476</v>
       </c>
       <c r="CE9" t="n">
-        <v>0.007239378611006459</v>
+        <v>0.007239378611006458</v>
       </c>
       <c r="CF9" t="n">
         <v>0.001276952497685258</v>
       </c>
       <c r="CG9" t="n">
-        <v>0.00430107127050358</v>
+        <v>0.004301071270503579</v>
       </c>
       <c r="CH9" t="n">
         <v>0.0005058538204923151</v>
@@ -5084,7 +5084,7 @@
         <v>0.000105131592714</v>
       </c>
       <c r="CJ9" t="n">
-        <v>0.007712362303394356</v>
+        <v>0.007712362303394358</v>
       </c>
       <c r="CK9" t="n">
         <v>9.298743096496996e-06</v>
@@ -5093,7 +5093,7 @@
         <v>0.0005142752676663607</v>
       </c>
       <c r="CM9" t="n">
-        <v>2.473825696082727e-05</v>
+        <v>2.473825696082728e-05</v>
       </c>
       <c r="CN9" t="n">
         <v>0.0002249550186030346</v>
@@ -5123,7 +5123,7 @@
         <v>0.0003829302297349509</v>
       </c>
       <c r="CW9" t="n">
-        <v>0.000431738207025463</v>
+        <v>0.0004317382070254632</v>
       </c>
       <c r="CX9" t="n">
         <v>0.004261356402639937</v>
@@ -5135,7 +5135,7 @@
         <v>0.0002605784200409152</v>
       </c>
       <c r="DA9" t="n">
-        <v>0.0003087262306103853</v>
+        <v>0.0003087262306103854</v>
       </c>
       <c r="DB9" t="n">
         <v>0.0005197055237990333</v>
@@ -5153,7 +5153,7 @@
         <v>0.0004720250126189642</v>
       </c>
       <c r="DG9" t="n">
-        <v>0.006020903563259797</v>
+        <v>0.006020903563259796</v>
       </c>
       <c r="DH9" t="n">
         <v>0.0005201630302955506</v>
@@ -5195,7 +5195,7 @@
         <v>0.001456093857529799</v>
       </c>
       <c r="DU9" t="n">
-        <v>0.003447447219291094</v>
+        <v>0.003447447219291095</v>
       </c>
       <c r="DV9" t="n">
         <v>9.4808575618102e-05</v>
@@ -5210,10 +5210,10 @@
         <v>0.0002644892628782009</v>
       </c>
       <c r="DZ9" t="n">
-        <v>0.0001980238905267614</v>
+        <v>0.0001980238905267615</v>
       </c>
       <c r="EA9" t="n">
-        <v>0.0004150350141639595</v>
+        <v>0.0004150350141639594</v>
       </c>
       <c r="EB9" t="n">
         <v>0.0002593212095877368</v>
@@ -5225,13 +5225,13 @@
         <v>9.643944624101786e-06</v>
       </c>
       <c r="EE9" t="n">
-        <v>7.360234912432838e-05</v>
+        <v>7.36023491243284e-05</v>
       </c>
       <c r="EF9" t="n">
         <v>3.842423521804625e-06</v>
       </c>
       <c r="EG9" t="n">
-        <v>6.86623352261418e-05</v>
+        <v>6.866233522614178e-05</v>
       </c>
       <c r="EH9" t="n">
         <v>3.434640813969186e-05</v>
@@ -5240,7 +5240,7 @@
         <v>2.587103487495073e-05</v>
       </c>
       <c r="EJ9" t="n">
-        <v>3.346903254062491e-05</v>
+        <v>3.346903254062493e-05</v>
       </c>
       <c r="EK9" t="n">
         <v>1.223260742146816</v>
@@ -5334,7 +5334,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>0.4224183149283154</v>
+        <v>0.4224183149283153</v>
       </c>
       <c r="C10" t="n">
         <v>0.0009731771207667348</v>
@@ -5346,10 +5346,10 @@
         <v>0.0125445729801706</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2424259790045787</v>
+        <v>0.2424259790045786</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5583310924903381</v>
+        <v>0.5583310924903379</v>
       </c>
       <c r="H10" t="n">
         <v>0.2668216473034422</v>
@@ -5367,22 +5367,22 @@
         <v>0.03610005043046514</v>
       </c>
       <c r="M10" t="n">
-        <v>0.006098691506406943</v>
+        <v>0.006098691506406944</v>
       </c>
       <c r="N10" t="n">
         <v>0.02146263184778546</v>
       </c>
       <c r="O10" t="n">
-        <v>0.004566701305922618</v>
+        <v>0.004566701305922619</v>
       </c>
       <c r="P10" t="n">
         <v>0.005843396852143966</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.007265777880520762</v>
+        <v>0.00726577788052076</v>
       </c>
       <c r="R10" t="n">
-        <v>0.007313670063244736</v>
+        <v>0.007313670063244735</v>
       </c>
       <c r="S10" t="n">
         <v>0.00515278328017468</v>
@@ -5394,7 +5394,7 @@
         <v>3.195283446445601e-05</v>
       </c>
       <c r="V10" t="n">
-        <v>0.001883565828390125</v>
+        <v>0.001883565828390124</v>
       </c>
       <c r="W10" t="n">
         <v>0.05245883400314946</v>
@@ -5406,25 +5406,25 @@
         <v>0.003936618385454477</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.003927550294526612</v>
+        <v>0.003927550294526613</v>
       </c>
       <c r="AA10" t="n">
-        <v>0.02331116474217443</v>
+        <v>0.02331116474217445</v>
       </c>
       <c r="AB10" t="n">
         <v>0.000880553244149592</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.03528452238758959</v>
+        <v>0.03528452238758958</v>
       </c>
       <c r="AD10" t="n">
-        <v>4.527773046452795e-05</v>
+        <v>4.527773046452794e-05</v>
       </c>
       <c r="AE10" t="n">
         <v>1.36001569327293e-05</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.05496989529383837</v>
+        <v>0.05496989529383833</v>
       </c>
       <c r="AG10" t="n">
         <v>0.03541799792337919</v>
@@ -5451,7 +5451,7 @@
         <v>0.0003062675937544332</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.0006193077142924304</v>
+        <v>0.0006193077142924301</v>
       </c>
       <c r="AP10" t="n">
         <v>0.0005079866712448635</v>
@@ -5460,7 +5460,7 @@
         <v>0.001583712811869542</v>
       </c>
       <c r="AR10" t="n">
-        <v>0.007491056713606628</v>
+        <v>0.007491056713606631</v>
       </c>
       <c r="AS10" t="n">
         <v>0.0001781226744022355</v>
@@ -5469,13 +5469,13 @@
         <v>8.850361794302431e-05</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.0003418303309742503</v>
+        <v>0.0003418303309742502</v>
       </c>
       <c r="AV10" t="n">
         <v>0.004250953948004395</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.003636454412703789</v>
+        <v>0.003636454412703787</v>
       </c>
       <c r="AX10" t="n">
         <v>0.0002690710198120019</v>
@@ -5490,28 +5490,28 @@
         <v>9.885941869999438e-05</v>
       </c>
       <c r="BB10" t="n">
-        <v>0.03905999606694455</v>
+        <v>0.03905999606694454</v>
       </c>
       <c r="BC10" t="n">
         <v>0.009626261157134294</v>
       </c>
       <c r="BD10" t="n">
-        <v>0.03246017506296604</v>
+        <v>0.03246017506296602</v>
       </c>
       <c r="BE10" t="n">
-        <v>0.0005062653919237684</v>
+        <v>0.0005062653919237685</v>
       </c>
       <c r="BF10" t="n">
         <v>0.0008451935192772085</v>
       </c>
       <c r="BG10" t="n">
-        <v>0.001105847097102291</v>
+        <v>0.00110584709710229</v>
       </c>
       <c r="BH10" t="n">
         <v>0.02053384157675798</v>
       </c>
       <c r="BI10" t="n">
-        <v>0.0004797574582327135</v>
+        <v>0.0004797574582327134</v>
       </c>
       <c r="BJ10" t="n">
         <v>1.390907258648706e-05</v>
@@ -5529,7 +5529,7 @@
         <v>0.001749536479925363</v>
       </c>
       <c r="BO10" t="n">
-        <v>6.85941196277827e-05</v>
+        <v>6.859411962778271e-05</v>
       </c>
       <c r="BP10" t="n">
         <v>0.0003012526461364932</v>
@@ -5571,7 +5571,7 @@
         <v>0.0003194197344847168</v>
       </c>
       <c r="CC10" t="n">
-        <v>0.0001197999713527573</v>
+        <v>0.0001197999713527574</v>
       </c>
       <c r="CD10" t="n">
         <v>0.000187088570063471</v>
@@ -5583,10 +5583,10 @@
         <v>0.001184034169540991</v>
       </c>
       <c r="CG10" t="n">
-        <v>0.00476733358663861</v>
+        <v>0.004767333586638608</v>
       </c>
       <c r="CH10" t="n">
-        <v>0.0004804863598406773</v>
+        <v>0.0004804863598406772</v>
       </c>
       <c r="CI10" t="n">
         <v>0.0001344048853553475</v>
@@ -5601,7 +5601,7 @@
         <v>0.0004718884182203335</v>
       </c>
       <c r="CM10" t="n">
-        <v>2.583608757101104e-05</v>
+        <v>2.583608757101105e-05</v>
       </c>
       <c r="CN10" t="n">
         <v>0.0002296812786545581</v>
@@ -5610,13 +5610,13 @@
         <v>0.00132904007450485</v>
       </c>
       <c r="CP10" t="n">
-        <v>0.0008654116170708709</v>
+        <v>0.0008654116170708716</v>
       </c>
       <c r="CQ10" t="n">
         <v>0.001126456309141461</v>
       </c>
       <c r="CR10" t="n">
-        <v>0.0006226681561362795</v>
+        <v>0.0006226681561362796</v>
       </c>
       <c r="CS10" t="n">
         <v>8.505491759945778e-05</v>
@@ -5631,7 +5631,7 @@
         <v>0.0003754577264816678</v>
       </c>
       <c r="CW10" t="n">
-        <v>0.0005011393458739696</v>
+        <v>0.0005011393458739697</v>
       </c>
       <c r="CX10" t="n">
         <v>0.004118925798625317</v>
@@ -5661,7 +5661,7 @@
         <v>0.0004822603137053306</v>
       </c>
       <c r="DG10" t="n">
-        <v>0.006207471292888288</v>
+        <v>0.006207471292888289</v>
       </c>
       <c r="DH10" t="n">
         <v>0.0004798137727617031</v>
@@ -5670,7 +5670,7 @@
         <v>8.508608771697038e-05</v>
       </c>
       <c r="DJ10" t="n">
-        <v>5.874514354711446e-05</v>
+        <v>5.874514354711443e-05</v>
       </c>
       <c r="DK10" t="n">
         <v>0.001132270706881733</v>
@@ -5679,16 +5679,16 @@
         <v>0.0002979893456883849</v>
       </c>
       <c r="DM10" t="n">
-        <v>0.0002095913366250654</v>
+        <v>0.0002095913366250653</v>
       </c>
       <c r="DN10" t="n">
-        <v>3.271250636896176e-05</v>
+        <v>3.271250636896177e-05</v>
       </c>
       <c r="DO10" t="n">
-        <v>0.001136243286093227</v>
+        <v>0.001136243286093226</v>
       </c>
       <c r="DP10" t="n">
-        <v>0.08525067786572045</v>
+        <v>0.08525067786572037</v>
       </c>
       <c r="DQ10" t="n">
         <v>7.702385588332861e-06</v>
@@ -5703,7 +5703,7 @@
         <v>0.001691869639363836</v>
       </c>
       <c r="DU10" t="n">
-        <v>0.003890576237390471</v>
+        <v>0.003890576237390472</v>
       </c>
       <c r="DV10" t="n">
         <v>8.564667677345881e-05</v>
@@ -5727,13 +5727,13 @@
         <v>0.000261828937378869</v>
       </c>
       <c r="EC10" t="n">
-        <v>0.005681897934782786</v>
+        <v>0.005681897934782785</v>
       </c>
       <c r="ED10" t="n">
         <v>7.725339143622216e-06</v>
       </c>
       <c r="EE10" t="n">
-        <v>7.27774545625532e-05</v>
+        <v>7.277745456255322e-05</v>
       </c>
       <c r="EF10" t="n">
         <v>4.567730043560163e-06</v>
@@ -5748,7 +5748,7 @@
         <v>2.794455247663429e-05</v>
       </c>
       <c r="EJ10" t="n">
-        <v>3.627131720215832e-05</v>
+        <v>3.627131720215831e-05</v>
       </c>
       <c r="EK10" t="n">
         <v>1.239796368527286</v>
@@ -5845,7 +5845,7 @@
         <v>0.3927613042226928</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0009001040096423594</v>
+        <v>0.0009001040096423587</v>
       </c>
       <c r="D11" t="n">
         <v>0.0008305757230112741</v>
@@ -5854,16 +5854,16 @@
         <v>0.01313612873128284</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2168672546525011</v>
+        <v>0.216867254652501</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5621063130926707</v>
+        <v>0.5621063130926715</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2271299957274628</v>
+        <v>0.227129995727463</v>
       </c>
       <c r="I11" t="n">
-        <v>0.06304588114846742</v>
+        <v>0.06304588114846743</v>
       </c>
       <c r="J11" t="n">
         <v>0.03050113451124808</v>
@@ -5878,13 +5878,13 @@
         <v>0.006119210245762084</v>
       </c>
       <c r="N11" t="n">
-        <v>0.02070635970999601</v>
+        <v>0.020706359709996</v>
       </c>
       <c r="O11" t="n">
         <v>0.004174605431637815</v>
       </c>
       <c r="P11" t="n">
-        <v>0.006219206048390012</v>
+        <v>0.00621920604839001</v>
       </c>
       <c r="Q11" t="n">
         <v>0.008609782022464625</v>
@@ -5893,7 +5893,7 @@
         <v>0.007130942413629641</v>
       </c>
       <c r="S11" t="n">
-        <v>0.005285492137918932</v>
+        <v>0.00528549213791893</v>
       </c>
       <c r="T11" t="n">
         <v>0.01571429964967858</v>
@@ -5908,43 +5908,43 @@
         <v>0.04213679849349709</v>
       </c>
       <c r="X11" t="n">
-        <v>0.0003713405638182861</v>
+        <v>0.0003713405638182862</v>
       </c>
       <c r="Y11" t="n">
         <v>0.00401253850174765</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.004022306898270746</v>
+        <v>0.004022306898270747</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.02799554354653958</v>
+        <v>0.0279955435465396</v>
       </c>
       <c r="AB11" t="n">
         <v>0.0008599745103255551</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.03443275662752716</v>
+        <v>0.03443275662752715</v>
       </c>
       <c r="AD11" t="n">
         <v>4.457734340344005e-05</v>
       </c>
       <c r="AE11" t="n">
-        <v>1.325747948049828e-05</v>
+        <v>1.325747948049829e-05</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.05760200694387686</v>
+        <v>0.05760200694387688</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.02849765431307863</v>
+        <v>0.02849765431307862</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.002064999519383479</v>
+        <v>0.002064999519383477</v>
       </c>
       <c r="AI11" t="n">
         <v>0.001330297068098717</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.002877478242600886</v>
+        <v>0.002877478242600884</v>
       </c>
       <c r="AK11" t="n">
         <v>0.0197396477769612</v>
@@ -5965,7 +5965,7 @@
         <v>0.0006170387923389534</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0.001570538545976575</v>
+        <v>0.001570538545976574</v>
       </c>
       <c r="AR11" t="n">
         <v>0.007605122230494715</v>
@@ -5980,7 +5980,7 @@
         <v>0.0003995464359297443</v>
       </c>
       <c r="AV11" t="n">
-        <v>0.003859721402552268</v>
+        <v>0.003859721402552269</v>
       </c>
       <c r="AW11" t="n">
         <v>0.003987252068719941</v>
@@ -5995,10 +5995,10 @@
         <v>0.0008122347629909497</v>
       </c>
       <c r="BA11" t="n">
-        <v>9.755652427636998e-05</v>
+        <v>9.75565242763699e-05</v>
       </c>
       <c r="BB11" t="n">
-        <v>0.03641294508856617</v>
+        <v>0.03641294508856615</v>
       </c>
       <c r="BC11" t="n">
         <v>0.008740826116006363</v>
@@ -6019,13 +6019,13 @@
         <v>0.01989926728436671</v>
       </c>
       <c r="BI11" t="n">
-        <v>0.0005153012396921023</v>
+        <v>0.0005153012396921024</v>
       </c>
       <c r="BJ11" t="n">
         <v>0.0001509650074374186</v>
       </c>
       <c r="BK11" t="n">
-        <v>0.01369892831667569</v>
+        <v>0.01369892831667568</v>
       </c>
       <c r="BL11" t="n">
         <v>8.280298130543375e-05</v>
@@ -6037,13 +6037,13 @@
         <v>0.00164696855611096</v>
       </c>
       <c r="BO11" t="n">
-        <v>6.250574451173411e-05</v>
+        <v>6.250574451173412e-05</v>
       </c>
       <c r="BP11" t="n">
         <v>0.0002834036871648271</v>
       </c>
       <c r="BQ11" t="n">
-        <v>0.0004762631390579144</v>
+        <v>0.0004762631390579143</v>
       </c>
       <c r="BR11" t="n">
         <v>0.0001912408626727468</v>
@@ -6052,7 +6052,7 @@
         <v>0.02689858911952969</v>
       </c>
       <c r="BT11" t="n">
-        <v>0.006102111442644785</v>
+        <v>0.006102111442644787</v>
       </c>
       <c r="BU11" t="n">
         <v>0.004013259743547977</v>
@@ -6064,7 +6064,7 @@
         <v>1.129186916551695e-05</v>
       </c>
       <c r="BX11" t="n">
-        <v>0.002555541814966951</v>
+        <v>0.00255554181496695</v>
       </c>
       <c r="BY11" t="n">
         <v>0.0001071546841740086</v>
@@ -6079,10 +6079,10 @@
         <v>0.0003208402555335389</v>
       </c>
       <c r="CC11" t="n">
-        <v>0.0001155254250924168</v>
+        <v>0.0001155254250924167</v>
       </c>
       <c r="CD11" t="n">
-        <v>0.0002536014918296583</v>
+        <v>0.0002536014918296584</v>
       </c>
       <c r="CE11" t="n">
         <v>0.007963372675573427</v>
@@ -6094,13 +6094,13 @@
         <v>0.004750916997842078</v>
       </c>
       <c r="CH11" t="n">
-        <v>0.0004762516942216756</v>
+        <v>0.0004762516942216757</v>
       </c>
       <c r="CI11" t="n">
         <v>0.0001211388013362684</v>
       </c>
       <c r="CJ11" t="n">
-        <v>0.008195279573858389</v>
+        <v>0.008195279573858382</v>
       </c>
       <c r="CK11" t="n">
         <v>9.34041368332001e-06</v>
@@ -6130,7 +6130,7 @@
         <v>0.0001044221102583587</v>
       </c>
       <c r="CT11" t="n">
-        <v>0.0002238461755984771</v>
+        <v>0.000223846175598477</v>
       </c>
       <c r="CU11" t="n">
         <v>0.0001153784751674855</v>
@@ -6169,10 +6169,10 @@
         <v>0.0004713688735576574</v>
       </c>
       <c r="DG11" t="n">
-        <v>0.005987424797261562</v>
+        <v>0.005987424797261561</v>
       </c>
       <c r="DH11" t="n">
-        <v>0.0004685544578870908</v>
+        <v>0.0004685544578870907</v>
       </c>
       <c r="DI11" t="n">
         <v>9.047099772942506e-05</v>
@@ -6205,7 +6205,7 @@
         <v>8.806277679587057e-05</v>
       </c>
       <c r="DS11" t="n">
-        <v>0.003519826232231614</v>
+        <v>0.003519826232231616</v>
       </c>
       <c r="DT11" t="n">
         <v>0.001563637756484061</v>
@@ -6350,28 +6350,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>0.3997486739716912</v>
+        <v>0.3997486739716914</v>
       </c>
       <c r="C12" t="n">
         <v>0.0009033436859297453</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0008795061911787017</v>
+        <v>0.000879506191178701</v>
       </c>
       <c r="E12" t="n">
         <v>0.01338985403059623</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2244592979384058</v>
+        <v>0.2244592979384059</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5587847287484471</v>
+        <v>0.5587847287484478</v>
       </c>
       <c r="H12" t="n">
         <v>0.2366756784218132</v>
       </c>
       <c r="I12" t="n">
-        <v>0.06437983001709734</v>
+        <v>0.06437983001709732</v>
       </c>
       <c r="J12" t="n">
         <v>0.02944351516413556</v>
@@ -6383,28 +6383,28 @@
         <v>0.03448166045904138</v>
       </c>
       <c r="M12" t="n">
-        <v>0.005467910157767718</v>
+        <v>0.005467910157767719</v>
       </c>
       <c r="N12" t="n">
-        <v>0.02010098911995819</v>
+        <v>0.0201009891199582</v>
       </c>
       <c r="O12" t="n">
-        <v>0.003947184133550462</v>
+        <v>0.003947184133550461</v>
       </c>
       <c r="P12" t="n">
-        <v>0.006140956599595907</v>
+        <v>0.006140956599595909</v>
       </c>
       <c r="Q12" t="n">
         <v>0.007863725633610657</v>
       </c>
       <c r="R12" t="n">
-        <v>0.006988193368375383</v>
+        <v>0.006988193368375382</v>
       </c>
       <c r="S12" t="n">
-        <v>0.005220563071132268</v>
+        <v>0.005220563071132269</v>
       </c>
       <c r="T12" t="n">
-        <v>0.01618095493951033</v>
+        <v>0.01618095493951034</v>
       </c>
       <c r="U12" t="n">
         <v>3.415047346663751e-05</v>
@@ -6413,22 +6413,22 @@
         <v>0.001898374748548179</v>
       </c>
       <c r="W12" t="n">
-        <v>0.04745493410170752</v>
+        <v>0.04745493410170753</v>
       </c>
       <c r="X12" t="n">
         <v>0.0004058413406473972</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.004015078534447647</v>
+        <v>0.004015078534447646</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.003835943853716995</v>
+        <v>0.003835943853716996</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.02751956947394898</v>
+        <v>0.02751956947394897</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.0009017637555758249</v>
+        <v>0.000901763755575824</v>
       </c>
       <c r="AC12" t="n">
         <v>0.03325049923838819</v>
@@ -6440,10 +6440,10 @@
         <v>1.332304912318154e-05</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.05977984331822755</v>
+        <v>0.05977984331822753</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.03035020629215674</v>
+        <v>0.03035020629215673</v>
       </c>
       <c r="AH12" t="n">
         <v>0.002019583431817152</v>
@@ -6455,22 +6455,22 @@
         <v>0.002768329354524335</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.0197297339094225</v>
+        <v>0.01972973390942251</v>
       </c>
       <c r="AL12" t="n">
         <v>0.0009143583335266284</v>
       </c>
       <c r="AM12" t="n">
-        <v>0.0003935483532908249</v>
+        <v>0.0003935483532908251</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.0003083494450859051</v>
+        <v>0.000308349445085905</v>
       </c>
       <c r="AO12" t="n">
         <v>0.0006290918541944786</v>
       </c>
       <c r="AP12" t="n">
-        <v>0.0005090088078499097</v>
+        <v>0.0005090088078499096</v>
       </c>
       <c r="AQ12" t="n">
         <v>0.001537502041263434</v>
@@ -6485,7 +6485,7 @@
         <v>8.176846637502431e-05</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.0003953813216756067</v>
+        <v>0.0003953813216756066</v>
       </c>
       <c r="AV12" t="n">
         <v>0.003968232090307461</v>
@@ -6497,28 +6497,28 @@
         <v>0.0003047866443877397</v>
       </c>
       <c r="AY12" t="n">
-        <v>0.03611871606269333</v>
+        <v>0.03611871606269332</v>
       </c>
       <c r="AZ12" t="n">
         <v>0.0008117901024291548</v>
       </c>
       <c r="BA12" t="n">
-        <v>9.967358397406388e-05</v>
+        <v>9.967358397406383e-05</v>
       </c>
       <c r="BB12" t="n">
-        <v>0.03813886188839966</v>
+        <v>0.03813886188839968</v>
       </c>
       <c r="BC12" t="n">
         <v>0.008957913426307779</v>
       </c>
       <c r="BD12" t="n">
-        <v>0.03347918221537487</v>
+        <v>0.03347918221537485</v>
       </c>
       <c r="BE12" t="n">
         <v>0.0005347441704871735</v>
       </c>
       <c r="BF12" t="n">
-        <v>0.0008449117668520585</v>
+        <v>0.0008449117668520592</v>
       </c>
       <c r="BG12" t="n">
         <v>0.001174644739498</v>
@@ -6533,13 +6533,13 @@
         <v>0.0001446075906485954</v>
       </c>
       <c r="BK12" t="n">
-        <v>0.01455330497681617</v>
+        <v>0.01455330497681616</v>
       </c>
       <c r="BL12" t="n">
         <v>8.362561340918776e-05</v>
       </c>
       <c r="BM12" t="n">
-        <v>0.02795911587176632</v>
+        <v>0.02795911587176633</v>
       </c>
       <c r="BN12" t="n">
         <v>0.001706782475754271</v>
@@ -6560,13 +6560,13 @@
         <v>0.02610345237148766</v>
       </c>
       <c r="BT12" t="n">
-        <v>0.005673609264695538</v>
+        <v>0.005673609264695536</v>
       </c>
       <c r="BU12" t="n">
         <v>0.003997431894849598</v>
       </c>
       <c r="BV12" t="n">
-        <v>0.003674748284135634</v>
+        <v>0.003674748284135635</v>
       </c>
       <c r="BW12" t="n">
         <v>9.17223735062505e-06</v>
@@ -6614,13 +6614,13 @@
         <v>1.001630004239213e-05</v>
       </c>
       <c r="CL12" t="n">
-        <v>0.0004998428177388662</v>
+        <v>0.0004998428177388663</v>
       </c>
       <c r="CM12" t="n">
         <v>2.943958849561442e-05</v>
       </c>
       <c r="CN12" t="n">
-        <v>0.0002564919588333966</v>
+        <v>0.0002564919588333965</v>
       </c>
       <c r="CO12" t="n">
         <v>0.001238610473057252</v>
@@ -6662,13 +6662,13 @@
         <v>0.0002953919780069211</v>
       </c>
       <c r="DB12" t="n">
-        <v>0.000509292126743105</v>
+        <v>0.0005092921267431049</v>
       </c>
       <c r="DC12" t="n">
         <v>0.0001120362953362746</v>
       </c>
       <c r="DD12" t="n">
-        <v>0.001446811132529484</v>
+        <v>0.001446811132529483</v>
       </c>
       <c r="DE12" t="n">
         <v>1.024279847932551e-05</v>
@@ -6686,7 +6686,7 @@
         <v>8.823100194475419e-05</v>
       </c>
       <c r="DJ12" t="n">
-        <v>6.358365978610061e-05</v>
+        <v>6.35836597861006e-05</v>
       </c>
       <c r="DK12" t="n">
         <v>0.001249280585944312</v>
@@ -6695,7 +6695,7 @@
         <v>0.0002821520781742289</v>
       </c>
       <c r="DM12" t="n">
-        <v>0.0001916480400660059</v>
+        <v>0.0001916480400660058</v>
       </c>
       <c r="DN12" t="n">
         <v>3.783204201062425e-05</v>
@@ -6704,19 +6704,19 @@
         <v>0.001102456084272922</v>
       </c>
       <c r="DP12" t="n">
-        <v>0.1062430045909735</v>
+        <v>0.1062430045909734</v>
       </c>
       <c r="DQ12" t="n">
         <v>7.526692992133471e-06</v>
       </c>
       <c r="DR12" t="n">
-        <v>8.144068699965362e-05</v>
+        <v>8.144068699965356e-05</v>
       </c>
       <c r="DS12" t="n">
         <v>0.003220020524857663</v>
       </c>
       <c r="DT12" t="n">
-        <v>0.001684303557023464</v>
+        <v>0.001684303557023463</v>
       </c>
       <c r="DU12" t="n">
         <v>0.003513568585081964</v>
@@ -6731,7 +6731,7 @@
         <v>0.0006968148020709399</v>
       </c>
       <c r="DY12" t="n">
-        <v>0.0002545918432439873</v>
+        <v>0.0002545918432439872</v>
       </c>
       <c r="DZ12" t="n">
         <v>0.0001922150708347241</v>
@@ -6740,7 +6740,7 @@
         <v>0.0004551043571077095</v>
       </c>
       <c r="EB12" t="n">
-        <v>0.0002667653291226905</v>
+        <v>0.0002667653291226906</v>
       </c>
       <c r="EC12" t="n">
         <v>0.00696434831213428</v>
@@ -6858,7 +6858,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>0.4029575683656931</v>
+        <v>0.4029575683656924</v>
       </c>
       <c r="C13" t="n">
         <v>0.0009911258553004885</v>
@@ -6876,7 +6876,7 @@
         <v>0.5466021605261879</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2295755366449047</v>
+        <v>0.2295755366449045</v>
       </c>
       <c r="I13" t="n">
         <v>0.05498120950354823</v>
@@ -6888,7 +6888,7 @@
         <v>0.07682420209201914</v>
       </c>
       <c r="L13" t="n">
-        <v>0.03661659824761725</v>
+        <v>0.03661659824761727</v>
       </c>
       <c r="M13" t="n">
         <v>0.006257835575850979</v>
@@ -6900,16 +6900,16 @@
         <v>0.004359834280795159</v>
       </c>
       <c r="P13" t="n">
-        <v>0.006429049964392364</v>
+        <v>0.006429049964392365</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.008751836352522835</v>
+        <v>0.008751836352522828</v>
       </c>
       <c r="R13" t="n">
-        <v>0.007199549184384033</v>
+        <v>0.007199549184384025</v>
       </c>
       <c r="S13" t="n">
-        <v>0.005439338367947628</v>
+        <v>0.005439338367947629</v>
       </c>
       <c r="T13" t="n">
         <v>0.01448361908764585</v>
@@ -6927,19 +6927,19 @@
         <v>0.0003764771683347946</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.004009560400312626</v>
+        <v>0.004009560400312625</v>
       </c>
       <c r="Z13" t="n">
         <v>0.004016066603758059</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.02772928275970316</v>
+        <v>0.02772928275970314</v>
       </c>
       <c r="AB13" t="n">
         <v>0.0008921494294329666</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.03547677419884859</v>
+        <v>0.03547677419884858</v>
       </c>
       <c r="AD13" t="n">
         <v>4.804965714772897e-05</v>
@@ -6951,10 +6951,10 @@
         <v>0.05554456905223483</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.03562610501758674</v>
+        <v>0.03562610501758675</v>
       </c>
       <c r="AH13" t="n">
-        <v>0.00201781924455335</v>
+        <v>0.002017819244553351</v>
       </c>
       <c r="AI13" t="n">
         <v>0.001271325317135847</v>
@@ -6978,7 +6978,7 @@
         <v>0.0006205032545987697</v>
       </c>
       <c r="AP13" t="n">
-        <v>0.0005454588007786162</v>
+        <v>0.0005454588007786163</v>
       </c>
       <c r="AQ13" t="n">
         <v>0.001590203900170766</v>
@@ -6990,10 +6990,10 @@
         <v>0.000158995723185645</v>
       </c>
       <c r="AT13" t="n">
-        <v>8.976213411041994e-05</v>
+        <v>8.976213411042001e-05</v>
       </c>
       <c r="AU13" t="n">
-        <v>0.0004219891390979902</v>
+        <v>0.0004219891390979903</v>
       </c>
       <c r="AV13" t="n">
         <v>0.003971715983529561</v>
@@ -7002,25 +7002,25 @@
         <v>0.004119756903385117</v>
       </c>
       <c r="AX13" t="n">
-        <v>0.0002919804776659674</v>
+        <v>0.0002919804776659676</v>
       </c>
       <c r="AY13" t="n">
-        <v>0.03357265576084898</v>
+        <v>0.03357265576084897</v>
       </c>
       <c r="AZ13" t="n">
         <v>0.0008646884872261088</v>
       </c>
       <c r="BA13" t="n">
-        <v>0.0001041830490403049</v>
+        <v>0.000104183049040305</v>
       </c>
       <c r="BB13" t="n">
-        <v>0.03938491367778248</v>
+        <v>0.03938491367778247</v>
       </c>
       <c r="BC13" t="n">
-        <v>0.008791296142347235</v>
+        <v>0.008791296142347227</v>
       </c>
       <c r="BD13" t="n">
-        <v>0.03554540556336339</v>
+        <v>0.03554540556336338</v>
       </c>
       <c r="BE13" t="n">
         <v>0.0005179800135510524</v>
@@ -7029,19 +7029,19 @@
         <v>0.0009205610883863398</v>
       </c>
       <c r="BG13" t="n">
-        <v>0.001127055979273568</v>
+        <v>0.001127055979273569</v>
       </c>
       <c r="BH13" t="n">
-        <v>0.02156003172107031</v>
+        <v>0.02156003172107032</v>
       </c>
       <c r="BI13" t="n">
-        <v>0.000522527477268284</v>
+        <v>0.0005225274772682841</v>
       </c>
       <c r="BJ13" t="n">
         <v>0.0002012482023852344</v>
       </c>
       <c r="BK13" t="n">
-        <v>0.01634725120525401</v>
+        <v>0.01634725120525402</v>
       </c>
       <c r="BL13" t="n">
         <v>8.584282646736607e-05</v>
@@ -7056,10 +7056,10 @@
         <v>6.63973715650966e-05</v>
       </c>
       <c r="BP13" t="n">
-        <v>0.0002943586909629766</v>
+        <v>0.0002943586909629767</v>
       </c>
       <c r="BQ13" t="n">
-        <v>0.0004847617474476743</v>
+        <v>0.0004847617474476742</v>
       </c>
       <c r="BR13" t="n">
         <v>0.0002024229207454696</v>
@@ -7068,13 +7068,13 @@
         <v>0.0293308497852251</v>
       </c>
       <c r="BT13" t="n">
-        <v>0.00559185346242362</v>
+        <v>0.005591853462423618</v>
       </c>
       <c r="BU13" t="n">
         <v>0.00399845249137139</v>
       </c>
       <c r="BV13" t="n">
-        <v>0.003813845155854458</v>
+        <v>0.003813845155854457</v>
       </c>
       <c r="BW13" t="n">
         <v>1.026281367244737e-05</v>
@@ -7095,7 +7095,7 @@
         <v>0.0003203667917502421</v>
       </c>
       <c r="CC13" t="n">
-        <v>0.0001286327593754401</v>
+        <v>0.0001286327593754402</v>
       </c>
       <c r="CD13" t="n">
         <v>0.0002217984292593931</v>
@@ -7110,7 +7110,7 @@
         <v>0.004935002338835611</v>
       </c>
       <c r="CH13" t="n">
-        <v>0.0005213264688691278</v>
+        <v>0.0005213264688691279</v>
       </c>
       <c r="CI13" t="n">
         <v>7.177216637475714e-05</v>
@@ -7140,19 +7140,19 @@
         <v>0.001069743228782819</v>
       </c>
       <c r="CR13" t="n">
-        <v>0.0006562119931608932</v>
+        <v>0.000656211993160893</v>
       </c>
       <c r="CS13" t="n">
         <v>0.0001014279990037085</v>
       </c>
       <c r="CT13" t="n">
-        <v>0.0002298527577265011</v>
+        <v>0.000229852757726501</v>
       </c>
       <c r="CU13" t="n">
         <v>0.0001213875442809819</v>
       </c>
       <c r="CV13" t="n">
-        <v>0.0004036414633258255</v>
+        <v>0.0004036414633258256</v>
       </c>
       <c r="CW13" t="n">
         <v>0.0004528579753936808</v>
@@ -7164,7 +7164,7 @@
         <v>0.0001402406437630826</v>
       </c>
       <c r="CZ13" t="n">
-        <v>0.0002891792640805329</v>
+        <v>0.000289179264080533</v>
       </c>
       <c r="DA13" t="n">
         <v>0.0003107929900444134</v>
@@ -7176,7 +7176,7 @@
         <v>0.0001038629239775857</v>
       </c>
       <c r="DD13" t="n">
-        <v>0.001541807274034559</v>
+        <v>0.00154180727403456</v>
       </c>
       <c r="DE13" t="n">
         <v>1.081516427792005e-05</v>
@@ -7185,16 +7185,16 @@
         <v>0.0004788199554279932</v>
       </c>
       <c r="DG13" t="n">
-        <v>0.005899227841421145</v>
+        <v>0.005899227841421142</v>
       </c>
       <c r="DH13" t="n">
-        <v>0.0004910635443756276</v>
+        <v>0.0004910635443756277</v>
       </c>
       <c r="DI13" t="n">
         <v>9.800187308532359e-05</v>
       </c>
       <c r="DJ13" t="n">
-        <v>5.044017312783787e-05</v>
+        <v>5.044017312783786e-05</v>
       </c>
       <c r="DK13" t="n">
         <v>0.001183688102568919</v>
@@ -7209,7 +7209,7 @@
         <v>3.965970970984978e-05</v>
       </c>
       <c r="DO13" t="n">
-        <v>0.001218568931624896</v>
+        <v>0.001218568931624897</v>
       </c>
       <c r="DP13" t="n">
         <v>0.09801641926546897</v>
@@ -7218,13 +7218,13 @@
         <v>7.802759505435844e-06</v>
       </c>
       <c r="DR13" t="n">
-        <v>0.0001010017483153961</v>
+        <v>0.0001010017483153962</v>
       </c>
       <c r="DS13" t="n">
-        <v>0.003505517034114726</v>
+        <v>0.003505517034114728</v>
       </c>
       <c r="DT13" t="n">
-        <v>0.001673859394140202</v>
+        <v>0.001673859394140203</v>
       </c>
       <c r="DU13" t="n">
         <v>0.003818084873973532</v>
@@ -7366,19 +7366,19 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>0.3745868375906418</v>
+        <v>0.3745868375906422</v>
       </c>
       <c r="C14" t="n">
         <v>0.0006606535057568974</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0007421043834532382</v>
+        <v>0.0007421043834532379</v>
       </c>
       <c r="E14" t="n">
         <v>0.01195299673536621</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2105056703590827</v>
+        <v>0.210505670359083</v>
       </c>
       <c r="G14" t="n">
         <v>0.5846018177044652</v>
@@ -7387,7 +7387,7 @@
         <v>0.2320566128257253</v>
       </c>
       <c r="I14" t="n">
-        <v>0.06705542245425808</v>
+        <v>0.06705542245425812</v>
       </c>
       <c r="J14" t="n">
         <v>0.02286413456756986</v>
@@ -7396,7 +7396,7 @@
         <v>0.0922941339980769</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0297605043280114</v>
+        <v>0.02976050432801141</v>
       </c>
       <c r="M14" t="n">
         <v>0.004351712635042238</v>
@@ -7408,7 +7408,7 @@
         <v>0.003369930334073482</v>
       </c>
       <c r="P14" t="n">
-        <v>0.004994654628512986</v>
+        <v>0.004994654628512982</v>
       </c>
       <c r="Q14" t="n">
         <v>0.004722456529650835</v>
@@ -7417,10 +7417,10 @@
         <v>0.006178693260952189</v>
       </c>
       <c r="S14" t="n">
-        <v>0.004280649971192278</v>
+        <v>0.004280649971192273</v>
       </c>
       <c r="T14" t="n">
-        <v>0.01627764605797259</v>
+        <v>0.01627764605797258</v>
       </c>
       <c r="U14" t="n">
         <v>2.745801347682813e-05</v>
@@ -7441,13 +7441,13 @@
         <v>0.003030284907741911</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.03345846546275212</v>
+        <v>0.03345846546275215</v>
       </c>
       <c r="AB14" t="n">
         <v>0.0007759001059731127</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.02724957836995043</v>
+        <v>0.02724957836995044</v>
       </c>
       <c r="AD14" t="n">
         <v>4.231279918826416e-05</v>
@@ -7468,7 +7468,7 @@
         <v>0.001347969863653445</v>
       </c>
       <c r="AJ14" t="n">
-        <v>0.002565134843833156</v>
+        <v>0.002565134843833155</v>
       </c>
       <c r="AK14" t="n">
         <v>0.01556563952171849</v>
@@ -7483,7 +7483,7 @@
         <v>0.0002685192756618342</v>
       </c>
       <c r="AO14" t="n">
-        <v>0.0005264138051664868</v>
+        <v>0.0005264138051664863</v>
       </c>
       <c r="AP14" t="n">
         <v>0.0003755585825982744</v>
@@ -7507,7 +7507,7 @@
         <v>0.003614099665546478</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.003430888200001615</v>
+        <v>0.003430888200001616</v>
       </c>
       <c r="AX14" t="n">
         <v>0.0002971737447005021</v>
@@ -7522,7 +7522,7 @@
         <v>7.519871835081359e-05</v>
       </c>
       <c r="BB14" t="n">
-        <v>0.0470618432799363</v>
+        <v>0.04706184327993634</v>
       </c>
       <c r="BC14" t="n">
         <v>0.007463279767988679</v>
@@ -7531,7 +7531,7 @@
         <v>0.02919181432732507</v>
       </c>
       <c r="BE14" t="n">
-        <v>0.0004445582881644009</v>
+        <v>0.0004445582881644006</v>
       </c>
       <c r="BF14" t="n">
         <v>0.0006965227743040091</v>
@@ -7540,7 +7540,7 @@
         <v>0.0009210921101643337</v>
       </c>
       <c r="BH14" t="n">
-        <v>0.0155214008746128</v>
+        <v>0.01552140087461281</v>
       </c>
       <c r="BI14" t="n">
         <v>0.0004020663068146826</v>
@@ -7549,7 +7549,7 @@
         <v>6.916426329507535e-06</v>
       </c>
       <c r="BK14" t="n">
-        <v>0.009325062347561235</v>
+        <v>0.009325062347561227</v>
       </c>
       <c r="BL14" t="n">
         <v>9.332807583133168e-05</v>
@@ -7561,7 +7561,7 @@
         <v>0.001543112532667671</v>
       </c>
       <c r="BO14" t="n">
-        <v>4.368069501540106e-05</v>
+        <v>4.36806950154011e-05</v>
       </c>
       <c r="BP14" t="n">
         <v>0.0002500667032105463</v>
@@ -7600,7 +7600,7 @@
         <v>0.0001005710406002073</v>
       </c>
       <c r="CB14" t="n">
-        <v>0.0002744632868822359</v>
+        <v>0.0002744632868822358</v>
       </c>
       <c r="CC14" t="n">
         <v>9.647610229423119e-05</v>
@@ -7690,7 +7690,7 @@
         <v>8.061391412552294e-06</v>
       </c>
       <c r="DF14" t="n">
-        <v>0.0003938557404281361</v>
+        <v>0.0003938557404281357</v>
       </c>
       <c r="DG14" t="n">
         <v>0.004876090302189321</v>
@@ -7717,10 +7717,10 @@
         <v>3.160777167259224e-05</v>
       </c>
       <c r="DO14" t="n">
-        <v>0.0009275555313592261</v>
+        <v>0.0009275555313592265</v>
       </c>
       <c r="DP14" t="n">
-        <v>0.1355465752808667</v>
+        <v>0.1355465752808668</v>
       </c>
       <c r="DQ14" t="n">
         <v>5.807179363487638e-06</v>
@@ -7744,7 +7744,7 @@
         <v>0.0003850057104404745</v>
       </c>
       <c r="DX14" t="n">
-        <v>0.0005644636656785762</v>
+        <v>0.0005644636656785766</v>
       </c>
       <c r="DY14" t="n">
         <v>0.0002291910798939039</v>
@@ -7756,7 +7756,7 @@
         <v>0.0003918527102783539</v>
       </c>
       <c r="EB14" t="n">
-        <v>0.0002267895913375495</v>
+        <v>0.0002267895913375494</v>
       </c>
       <c r="EC14" t="n">
         <v>0.007676321166441735</v>
@@ -7874,7 +7874,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>0.3742668276483801</v>
+        <v>0.3742668276483794</v>
       </c>
       <c r="C15" t="n">
         <v>0.0006769301927890275</v>
@@ -7886,13 +7886,13 @@
         <v>0.01251693699455387</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2110347464309044</v>
+        <v>0.2110347464309048</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5819908750752426</v>
+        <v>0.5819908750752433</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2295379752627645</v>
+        <v>0.2295379752627642</v>
       </c>
       <c r="I15" t="n">
         <v>0.06368476116144381</v>
@@ -7904,7 +7904,7 @@
         <v>0.09208671485886526</v>
       </c>
       <c r="L15" t="n">
-        <v>0.03019627805468142</v>
+        <v>0.03019627805468141</v>
       </c>
       <c r="M15" t="n">
         <v>0.004026277802644333</v>
@@ -7919,16 +7919,16 @@
         <v>0.004854955675197013</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.006061649686325234</v>
+        <v>0.006061649686325238</v>
       </c>
       <c r="R15" t="n">
         <v>0.006222076046113688</v>
       </c>
       <c r="S15" t="n">
-        <v>0.004352289928152074</v>
+        <v>0.004352289928152078</v>
       </c>
       <c r="T15" t="n">
-        <v>0.01585275927729118</v>
+        <v>0.01585275927729119</v>
       </c>
       <c r="U15" t="n">
         <v>2.747479263017608e-05</v>
@@ -7937,7 +7937,7 @@
         <v>0.001603428814634244</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04799296143579568</v>
+        <v>0.04799296143579572</v>
       </c>
       <c r="X15" t="n">
         <v>0.0003725669646492275</v>
@@ -7946,16 +7946,16 @@
         <v>0.003622164216168038</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.00293400925960779</v>
+        <v>0.002934009259607789</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.03532218685848586</v>
+        <v>0.03532218685848585</v>
       </c>
       <c r="AB15" t="n">
         <v>0.0007351061333116742</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.02762012487575338</v>
+        <v>0.0276201248757534</v>
       </c>
       <c r="AD15" t="n">
         <v>4.38334204413744e-05</v>
@@ -8018,7 +8018,7 @@
         <v>0.004158442541142755</v>
       </c>
       <c r="AX15" t="n">
-        <v>0.0003008556130213227</v>
+        <v>0.0003008556130213228</v>
       </c>
       <c r="AY15" t="n">
         <v>0.04587665502870054</v>
@@ -8033,7 +8033,7 @@
         <v>0.04325090906327643</v>
       </c>
       <c r="BC15" t="n">
-        <v>0.007276488646914736</v>
+        <v>0.007276488646914732</v>
       </c>
       <c r="BD15" t="n">
         <v>0.02802716304497264</v>
@@ -8048,7 +8048,7 @@
         <v>0.0009797499173313465</v>
       </c>
       <c r="BH15" t="n">
-        <v>0.01506785459261033</v>
+        <v>0.01506785459261034</v>
       </c>
       <c r="BI15" t="n">
         <v>0.0004403800931488896</v>
@@ -8090,7 +8090,7 @@
         <v>0.003272191200050852</v>
       </c>
       <c r="BV15" t="n">
-        <v>0.003408138637985754</v>
+        <v>0.003408138637985755</v>
       </c>
       <c r="BW15" t="n">
         <v>6.291442630911805e-06</v>
@@ -8105,7 +8105,7 @@
         <v>0.004599006275810364</v>
       </c>
       <c r="CA15" t="n">
-        <v>9.980536536734841e-05</v>
+        <v>9.980536536734845e-05</v>
       </c>
       <c r="CB15" t="n">
         <v>0.0003215918056576125</v>
@@ -8120,7 +8120,7 @@
         <v>0.008436647723431433</v>
       </c>
       <c r="CF15" t="n">
-        <v>0.001464901281796551</v>
+        <v>0.001464901281796552</v>
       </c>
       <c r="CG15" t="n">
         <v>0.002878440557859495</v>
@@ -8138,7 +8138,7 @@
         <v>9.072213996944829e-06</v>
       </c>
       <c r="CL15" t="n">
-        <v>0.0003819229468996528</v>
+        <v>0.0003819229468996525</v>
       </c>
       <c r="CM15" t="n">
         <v>2.36763084507809e-05</v>
@@ -8156,7 +8156,7 @@
         <v>0.0007792519032442457</v>
       </c>
       <c r="CR15" t="n">
-        <v>0.0005634966491209872</v>
+        <v>0.0005634966491209869</v>
       </c>
       <c r="CS15" t="n">
         <v>0.0001031149742182792</v>
@@ -8174,7 +8174,7 @@
         <v>0.0004129523555838243</v>
       </c>
       <c r="CX15" t="n">
-        <v>0.003594849254041952</v>
+        <v>0.003594849254041951</v>
       </c>
       <c r="CY15" t="n">
         <v>0.0001051140167921165</v>
@@ -8198,7 +8198,7 @@
         <v>7.839394225268833e-06</v>
       </c>
       <c r="DF15" t="n">
-        <v>0.0004317813060713909</v>
+        <v>0.0004317813060713912</v>
       </c>
       <c r="DG15" t="n">
         <v>0.004799503675923678</v>
@@ -8228,7 +8228,7 @@
         <v>0.00097493685741852</v>
       </c>
       <c r="DP15" t="n">
-        <v>0.1346390487985742</v>
+        <v>0.1346390487985743</v>
       </c>
       <c r="DQ15" t="n">
         <v>5.04801871112189e-06</v>
@@ -8246,7 +8246,7 @@
         <v>0.003009452438792379</v>
       </c>
       <c r="DV15" t="n">
-        <v>5.360459942496808e-05</v>
+        <v>5.360459942496804e-05</v>
       </c>
       <c r="DW15" t="n">
         <v>0.0003842562965751591</v>
@@ -8264,7 +8264,7 @@
         <v>0.0003818068117353458</v>
       </c>
       <c r="EB15" t="n">
-        <v>0.000233287762554817</v>
+        <v>0.0002332877625548169</v>
       </c>
       <c r="EC15" t="n">
         <v>0.007193331111141901</v>
@@ -8273,7 +8273,7 @@
         <v>6.953013573797032e-06</v>
       </c>
       <c r="EE15" t="n">
-        <v>8.843325095809088e-05</v>
+        <v>8.843325095809092e-05</v>
       </c>
       <c r="EF15" t="n">
         <v>2.528636188503109e-06</v>
@@ -8382,7 +8382,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>0.3657186585318448</v>
+        <v>0.3657186585318444</v>
       </c>
       <c r="C16" t="n">
         <v>0.000683673684086022</v>
@@ -8394,16 +8394,16 @@
         <v>0.01152061079266303</v>
       </c>
       <c r="F16" t="n">
-        <v>0.2127694780042606</v>
+        <v>0.2127694780042605</v>
       </c>
       <c r="G16" t="n">
         <v>0.5904443920865803</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2363497748289705</v>
+        <v>0.2363497748289704</v>
       </c>
       <c r="I16" t="n">
-        <v>0.07416612364991566</v>
+        <v>0.07416612364991571</v>
       </c>
       <c r="J16" t="n">
         <v>0.02424358493697039</v>
@@ -8433,10 +8433,10 @@
         <v>0.006222182609674423</v>
       </c>
       <c r="S16" t="n">
-        <v>0.004442398884272197</v>
+        <v>0.004442398884272193</v>
       </c>
       <c r="T16" t="n">
-        <v>0.01583746084156089</v>
+        <v>0.01583746084156087</v>
       </c>
       <c r="U16" t="n">
         <v>2.995293942142188e-05</v>
@@ -8457,7 +8457,7 @@
         <v>0.003151270616164604</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.03415193149873701</v>
+        <v>0.03415193149873699</v>
       </c>
       <c r="AB16" t="n">
         <v>0.0007439409127351945</v>
@@ -8487,7 +8487,7 @@
         <v>0.002831662998598645</v>
       </c>
       <c r="AK16" t="n">
-        <v>0.01489156401294473</v>
+        <v>0.01489156401294472</v>
       </c>
       <c r="AL16" t="n">
         <v>0.0008335158693714261</v>
@@ -8526,22 +8526,22 @@
         <v>0.003631080257650435</v>
       </c>
       <c r="AX16" t="n">
-        <v>0.00031333220723601</v>
+        <v>0.0003133322072360099</v>
       </c>
       <c r="AY16" t="n">
         <v>0.04765013814228587</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0.0006409902506775121</v>
+        <v>0.0006409902506775118</v>
       </c>
       <c r="BA16" t="n">
         <v>7.720283711517966e-05</v>
       </c>
       <c r="BB16" t="n">
-        <v>0.0449431200457082</v>
+        <v>0.04494312004570824</v>
       </c>
       <c r="BC16" t="n">
-        <v>0.007289456104182892</v>
+        <v>0.007289456104182888</v>
       </c>
       <c r="BD16" t="n">
         <v>0.02609169648087678</v>
@@ -8553,7 +8553,7 @@
         <v>0.0007424728586599112</v>
       </c>
       <c r="BG16" t="n">
-        <v>0.0009463407274249001</v>
+        <v>0.0009463407274248998</v>
       </c>
       <c r="BH16" t="n">
         <v>0.01662528403657262</v>
@@ -8568,7 +8568,7 @@
         <v>0.008325147604889659</v>
       </c>
       <c r="BL16" t="n">
-        <v>8.271855164940514e-05</v>
+        <v>8.27185516494052e-05</v>
       </c>
       <c r="BM16" t="n">
         <v>0.02385791986934216</v>
@@ -8589,7 +8589,7 @@
         <v>0.0001003335179018672</v>
       </c>
       <c r="BS16" t="n">
-        <v>0.01950772879508408</v>
+        <v>0.01950772879508409</v>
       </c>
       <c r="BT16" t="n">
         <v>0.005707164836676754</v>
@@ -8604,7 +8604,7 @@
         <v>7.759009356925431e-06</v>
       </c>
       <c r="BX16" t="n">
-        <v>0.002371626641604716</v>
+        <v>0.002371626641604717</v>
       </c>
       <c r="BY16" t="n">
         <v>0.0001260782076456296</v>
@@ -8634,7 +8634,7 @@
         <v>0.003057060948564139</v>
       </c>
       <c r="CH16" t="n">
-        <v>0.0003956386348537367</v>
+        <v>0.000395638634853737</v>
       </c>
       <c r="CI16" t="n">
         <v>0.0001455378523668287</v>
@@ -8658,7 +8658,7 @@
         <v>0.0005476144445495923</v>
       </c>
       <c r="CP16" t="n">
-        <v>0.000590924900313925</v>
+        <v>0.0005909249003139253</v>
       </c>
       <c r="CQ16" t="n">
         <v>0.0006230567426738979</v>
@@ -8673,10 +8673,10 @@
         <v>0.0002041728062131509</v>
       </c>
       <c r="CU16" t="n">
-        <v>0.000106927666878267</v>
+        <v>0.0001069276668782671</v>
       </c>
       <c r="CV16" t="n">
-        <v>0.0003274659057504117</v>
+        <v>0.0003274659057504116</v>
       </c>
       <c r="CW16" t="n">
         <v>0.0003671049326700668</v>
@@ -8685,7 +8685,7 @@
         <v>0.00279219894633889</v>
       </c>
       <c r="CY16" t="n">
-        <v>0.0001135633171057593</v>
+        <v>0.0001135633171057592</v>
       </c>
       <c r="CZ16" t="n">
         <v>0.000213814215210132</v>
@@ -8709,10 +8709,10 @@
         <v>0.0003352321035562029</v>
       </c>
       <c r="DG16" t="n">
-        <v>0.004840394505408675</v>
+        <v>0.004840394505408672</v>
       </c>
       <c r="DH16" t="n">
-        <v>0.0004541330741694497</v>
+        <v>0.0004541330741694502</v>
       </c>
       <c r="DI16" t="n">
         <v>9.054859350222305e-05</v>
@@ -8724,10 +8724,10 @@
         <v>0.001138868875978576</v>
       </c>
       <c r="DL16" t="n">
-        <v>0.0002297292812005106</v>
+        <v>0.0002297292812005107</v>
       </c>
       <c r="DM16" t="n">
-        <v>0.000209133756394277</v>
+        <v>0.0002091337563942769</v>
       </c>
       <c r="DN16" t="n">
         <v>3.702142003373666e-05</v>
@@ -8781,7 +8781,7 @@
         <v>5.568413747252949e-06</v>
       </c>
       <c r="EE16" t="n">
-        <v>9.188427525466688e-05</v>
+        <v>9.188427525466684e-05</v>
       </c>
       <c r="EF16" t="n">
         <v>2.345319811165469e-06</v>
@@ -8790,7 +8790,7 @@
         <v>5.938930979330267e-05</v>
       </c>
       <c r="EH16" t="n">
-        <v>3.498908955599258e-05</v>
+        <v>3.498908955599257e-05</v>
       </c>
       <c r="EI16" t="n">
         <v>2.73519475480262e-05</v>
@@ -8890,25 +8890,25 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>0.3592142414100321</v>
+        <v>0.3592142414100323</v>
       </c>
       <c r="C17" t="n">
         <v>0.0005797234571972056</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0006767661585358676</v>
+        <v>0.000676766158535867</v>
       </c>
       <c r="E17" t="n">
         <v>0.01032920301830001</v>
       </c>
       <c r="F17" t="n">
-        <v>0.2148342306962203</v>
+        <v>0.2148342306962207</v>
       </c>
       <c r="G17" t="n">
         <v>0.6093015405986165</v>
       </c>
       <c r="H17" t="n">
-        <v>0.2434412493288412</v>
+        <v>0.2434412493288413</v>
       </c>
       <c r="I17" t="n">
         <v>0.07707292660978328</v>
@@ -8920,31 +8920,31 @@
         <v>0.1014235631803267</v>
       </c>
       <c r="L17" t="n">
-        <v>0.02616500361033504</v>
+        <v>0.02616500361033503</v>
       </c>
       <c r="M17" t="n">
-        <v>0.002898387044709068</v>
+        <v>0.002898387044709071</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0126434414871194</v>
+        <v>0.01264344148711941</v>
       </c>
       <c r="O17" t="n">
         <v>0.00305907635596417</v>
       </c>
       <c r="P17" t="n">
-        <v>0.00436210476141869</v>
+        <v>0.004362104761418687</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.004671378986097246</v>
+        <v>0.004671378986097249</v>
       </c>
       <c r="R17" t="n">
-        <v>0.005722387961358265</v>
+        <v>0.005722387961358269</v>
       </c>
       <c r="S17" t="n">
-        <v>0.004088979659470145</v>
+        <v>0.004088979659470148</v>
       </c>
       <c r="T17" t="n">
-        <v>0.01490157043620636</v>
+        <v>0.01490157043620637</v>
       </c>
       <c r="U17" t="n">
         <v>2.865218104956496e-05</v>
@@ -8956,13 +8956,13 @@
         <v>0.04779620990327637</v>
       </c>
       <c r="X17" t="n">
-        <v>0.0003199810516451335</v>
+        <v>0.0003199810516451339</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.003138312495932897</v>
+        <v>0.003138312495932894</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.002655807928927975</v>
+        <v>0.002655807928927974</v>
       </c>
       <c r="AA17" t="n">
         <v>0.03762579335559059</v>
@@ -8971,7 +8971,7 @@
         <v>0.0006412815292484092</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.0235267407597898</v>
+        <v>0.02352674075978979</v>
       </c>
       <c r="AD17" t="n">
         <v>4.343386356842002e-05</v>
@@ -8986,13 +8986,13 @@
         <v>0.02375014221362074</v>
       </c>
       <c r="AH17" t="n">
-        <v>0.001904074238955246</v>
+        <v>0.001904074238955245</v>
       </c>
       <c r="AI17" t="n">
         <v>0.001090060926815166</v>
       </c>
       <c r="AJ17" t="n">
-        <v>0.002363998258749109</v>
+        <v>0.00236399825874911</v>
       </c>
       <c r="AK17" t="n">
         <v>0.0132878048555289</v>
@@ -9037,7 +9037,7 @@
         <v>0.0002829044346950708</v>
       </c>
       <c r="AY17" t="n">
-        <v>0.05359375051953088</v>
+        <v>0.05359375051953085</v>
       </c>
       <c r="AZ17" t="n">
         <v>0.000552082732991472</v>
@@ -9049,10 +9049,10 @@
         <v>0.04886657998433273</v>
       </c>
       <c r="BC17" t="n">
-        <v>0.006804386168348159</v>
+        <v>0.006804386168348163</v>
       </c>
       <c r="BD17" t="n">
-        <v>0.02214202986634855</v>
+        <v>0.02214202986634854</v>
       </c>
       <c r="BE17" t="n">
         <v>0.000383400056248179</v>
@@ -9088,7 +9088,7 @@
         <v>3.790217554829133e-05</v>
       </c>
       <c r="BP17" t="n">
-        <v>0.0002080555588645427</v>
+        <v>0.0002080555588645426</v>
       </c>
       <c r="BQ17" t="n">
         <v>0.0004929698411740952</v>
@@ -9100,7 +9100,7 @@
         <v>0.01681993792424363</v>
       </c>
       <c r="BT17" t="n">
-        <v>0.005939143501909484</v>
+        <v>0.005939143501909487</v>
       </c>
       <c r="BU17" t="n">
         <v>0.002702769091263287</v>
@@ -9112,22 +9112,22 @@
         <v>5.050147252675561e-06</v>
       </c>
       <c r="BX17" t="n">
-        <v>0.002042727213716987</v>
+        <v>0.002042727213716986</v>
       </c>
       <c r="BY17" t="n">
         <v>0.000104682592842036</v>
       </c>
       <c r="BZ17" t="n">
-        <v>0.003408499243218248</v>
+        <v>0.003408499243218245</v>
       </c>
       <c r="CA17" t="n">
-        <v>8.635270826925171e-05</v>
+        <v>8.635270826925168e-05</v>
       </c>
       <c r="CB17" t="n">
         <v>0.0003294409049942673</v>
       </c>
       <c r="CC17" t="n">
-        <v>8.472291645198791e-05</v>
+        <v>8.472291645198798e-05</v>
       </c>
       <c r="CD17" t="n">
         <v>0.0001626668326362286</v>
@@ -9139,7 +9139,7 @@
         <v>0.001249841231396708</v>
       </c>
       <c r="CG17" t="n">
-        <v>0.001971092077951117</v>
+        <v>0.001971092077951116</v>
       </c>
       <c r="CH17" t="n">
         <v>0.0003664682219733398</v>
@@ -9163,16 +9163,16 @@
         <v>0.0002209741481720769</v>
       </c>
       <c r="CO17" t="n">
-        <v>0.0009520600251581215</v>
+        <v>0.0009520600251581208</v>
       </c>
       <c r="CP17" t="n">
         <v>0.0005674705423025673</v>
       </c>
       <c r="CQ17" t="n">
-        <v>0.000570432586830578</v>
+        <v>0.0005704325868305784</v>
       </c>
       <c r="CR17" t="n">
-        <v>0.0005544443176426115</v>
+        <v>0.0005544443176426118</v>
       </c>
       <c r="CS17" t="n">
         <v>8.866520999326356e-05</v>
@@ -9211,7 +9211,7 @@
         <v>0.001069807747485388</v>
       </c>
       <c r="DE17" t="n">
-        <v>6.873481766846091e-06</v>
+        <v>6.873481766846088e-06</v>
       </c>
       <c r="DF17" t="n">
         <v>0.0003679999278624259</v>
@@ -9398,7 +9398,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>0.3650342009336014</v>
+        <v>0.3650342009336016</v>
       </c>
       <c r="C18" t="n">
         <v>0.0005696592021732335</v>
@@ -9410,13 +9410,13 @@
         <v>0.01020828125458456</v>
       </c>
       <c r="F18" t="n">
-        <v>0.2217892661567526</v>
+        <v>0.2217892661567525</v>
       </c>
       <c r="G18" t="n">
-        <v>0.6105417468267413</v>
+        <v>0.610541746826741</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2585679992503967</v>
+        <v>0.2585679992503968</v>
       </c>
       <c r="I18" t="n">
         <v>0.0810766574926836</v>
@@ -9443,13 +9443,13 @@
         <v>0.004274422958892725</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.004481745631244778</v>
+        <v>0.004481745631244775</v>
       </c>
       <c r="R18" t="n">
         <v>0.006512777118788152</v>
       </c>
       <c r="S18" t="n">
-        <v>0.004019155835911671</v>
+        <v>0.004019155835911675</v>
       </c>
       <c r="T18" t="n">
         <v>0.01323227985844572</v>
@@ -9458,13 +9458,13 @@
         <v>2.868418450260135e-05</v>
       </c>
       <c r="V18" t="n">
-        <v>0.001366137459076177</v>
+        <v>0.001366137459076176</v>
       </c>
       <c r="W18" t="n">
         <v>0.05871949883175197</v>
       </c>
       <c r="X18" t="n">
-        <v>0.0003400470523882176</v>
+        <v>0.000340047052388218</v>
       </c>
       <c r="Y18" t="n">
         <v>0.003074300827190869</v>
@@ -9479,22 +9479,22 @@
         <v>0.0006198666288863056</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.02275738719670906</v>
+        <v>0.02275738719670907</v>
       </c>
       <c r="AD18" t="n">
         <v>2.7527559007701e-05</v>
       </c>
       <c r="AE18" t="n">
-        <v>8.00412023892052e-06</v>
+        <v>8.004120238920518e-06</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.06692209692445332</v>
+        <v>0.06692209692445335</v>
       </c>
       <c r="AG18" t="n">
-        <v>0.02280353246081933</v>
+        <v>0.02280353246081934</v>
       </c>
       <c r="AH18" t="n">
-        <v>0.001856459899621282</v>
+        <v>0.001856459899621281</v>
       </c>
       <c r="AI18" t="n">
         <v>0.001174407523124253</v>
@@ -9506,7 +9506,7 @@
         <v>0.01164600652073184</v>
       </c>
       <c r="AL18" t="n">
-        <v>0.0006893096633073772</v>
+        <v>0.0006893096633073769</v>
       </c>
       <c r="AM18" t="n">
         <v>0.0002643910998764151</v>
@@ -9524,7 +9524,7 @@
         <v>0.00130025567812156</v>
       </c>
       <c r="AR18" t="n">
-        <v>0.006760586455906059</v>
+        <v>0.006760586455906063</v>
       </c>
       <c r="AS18" t="n">
         <v>0.0001540966347736209</v>
@@ -9533,7 +9533,7 @@
         <v>4.363284252150871e-05</v>
       </c>
       <c r="AU18" t="n">
-        <v>0.0002657731735858922</v>
+        <v>0.0002657731735858921</v>
       </c>
       <c r="AV18" t="n">
         <v>0.003935888420612569</v>
@@ -9548,19 +9548,19 @@
         <v>0.0552111968303122</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0.0005271878128941191</v>
+        <v>0.0005271878128941193</v>
       </c>
       <c r="BA18" t="n">
         <v>6.214241074019171e-05</v>
       </c>
       <c r="BB18" t="n">
-        <v>0.05022123900681674</v>
+        <v>0.05022123900681676</v>
       </c>
       <c r="BC18" t="n">
-        <v>0.006784337228342121</v>
+        <v>0.006784337228342118</v>
       </c>
       <c r="BD18" t="n">
-        <v>0.02323241079605995</v>
+        <v>0.02323241079605992</v>
       </c>
       <c r="BE18" t="n">
         <v>0.0004180363681211612</v>
@@ -9572,7 +9572,7 @@
         <v>0.0007142882419329292</v>
       </c>
       <c r="BH18" t="n">
-        <v>0.01410614445461149</v>
+        <v>0.01410614445461148</v>
       </c>
       <c r="BI18" t="n">
         <v>0.0004348511587189965</v>
@@ -9581,7 +9581,7 @@
         <v>2.231561562412052e-06</v>
       </c>
       <c r="BK18" t="n">
-        <v>0.007716306227240419</v>
+        <v>0.007716306227240415</v>
       </c>
       <c r="BL18" t="n">
         <v>8.853941025930571e-05</v>
@@ -9608,7 +9608,7 @@
         <v>0.01668610559968934</v>
       </c>
       <c r="BT18" t="n">
-        <v>0.004829788899865069</v>
+        <v>0.004829788899865072</v>
       </c>
       <c r="BU18" t="n">
         <v>0.002561413536539373</v>
@@ -9686,7 +9686,7 @@
         <v>8.735176577761552e-05</v>
       </c>
       <c r="CT18" t="n">
-        <v>0.0001663489749297676</v>
+        <v>0.0001663489749297677</v>
       </c>
       <c r="CU18" t="n">
         <v>8.839561430257429e-05</v>
@@ -9725,7 +9725,7 @@
         <v>0.00045197793748535</v>
       </c>
       <c r="DG18" t="n">
-        <v>0.004317910988237221</v>
+        <v>0.004317910988237223</v>
       </c>
       <c r="DH18" t="n">
         <v>0.0003997466693822759</v>
@@ -9737,7 +9737,7 @@
         <v>4.505278407876487e-05</v>
       </c>
       <c r="DK18" t="n">
-        <v>0.001024469082008705</v>
+        <v>0.001024469082008704</v>
       </c>
       <c r="DL18" t="n">
         <v>0.000178331775078999</v>
@@ -9779,7 +9779,7 @@
         <v>0.0005041738044867757</v>
       </c>
       <c r="DY18" t="n">
-        <v>0.0002369804197105962</v>
+        <v>0.0002369804197105963</v>
       </c>
       <c r="DZ18" t="n">
         <v>0.0001603662093148674</v>
@@ -9803,7 +9803,7 @@
         <v>1.745565880593482e-06</v>
       </c>
       <c r="EG18" t="n">
-        <v>4.504922890370274e-05</v>
+        <v>4.504922890370271e-05</v>
       </c>
       <c r="EH18" t="n">
         <v>2.720933235499135e-05</v>
@@ -9918,10 +9918,10 @@
         <v>0.01030822963792791</v>
       </c>
       <c r="F19" t="n">
-        <v>0.2099842098305724</v>
+        <v>0.2099842098305725</v>
       </c>
       <c r="G19" t="n">
-        <v>0.6027095015948645</v>
+        <v>0.6027095015948652</v>
       </c>
       <c r="H19" t="n">
         <v>0.2402872979684584</v>
@@ -9936,7 +9936,7 @@
         <v>0.1001814109343353</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0279510647360637</v>
+        <v>0.02795106473606373</v>
       </c>
       <c r="M19" t="n">
         <v>0.00331706862130119</v>
@@ -9948,7 +9948,7 @@
         <v>0.003148384273029454</v>
       </c>
       <c r="P19" t="n">
-        <v>0.004622816887055404</v>
+        <v>0.004622816887055406</v>
       </c>
       <c r="Q19" t="n">
         <v>0.004965720391699337</v>
@@ -9984,7 +9984,7 @@
         <v>0.03816464914869597</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.0006626274530067977</v>
+        <v>0.0006626274530067974</v>
       </c>
       <c r="AC19" t="n">
         <v>0.02520750419250734</v>
@@ -9993,19 +9993,19 @@
         <v>2.818519636219284e-05</v>
       </c>
       <c r="AE19" t="n">
-        <v>9.968723616546825e-06</v>
+        <v>9.968723616546827e-06</v>
       </c>
       <c r="AF19" t="n">
-        <v>0.06379879681704455</v>
+        <v>0.06379879681704456</v>
       </c>
       <c r="AG19" t="n">
         <v>0.02356429643839769</v>
       </c>
       <c r="AH19" t="n">
-        <v>0.001820519767030029</v>
+        <v>0.001820519767030028</v>
       </c>
       <c r="AI19" t="n">
-        <v>0.001225896456566014</v>
+        <v>0.001225896456566013</v>
       </c>
       <c r="AJ19" t="n">
         <v>0.002579585357292189</v>
@@ -10017,7 +10017,7 @@
         <v>0.0007091833770896643</v>
       </c>
       <c r="AM19" t="n">
-        <v>0.0003003048909164891</v>
+        <v>0.0003003048909164887</v>
       </c>
       <c r="AN19" t="n">
         <v>0.0002605632195647156</v>
@@ -10035,7 +10035,7 @@
         <v>0.007062580459950529</v>
       </c>
       <c r="AS19" t="n">
-        <v>0.000150788777677652</v>
+        <v>0.0001507887776776519</v>
       </c>
       <c r="AT19" t="n">
         <v>5.619932723971792e-05</v>
@@ -10065,10 +10065,10 @@
         <v>0.05010367791298082</v>
       </c>
       <c r="BC19" t="n">
-        <v>0.006800807162446394</v>
+        <v>0.006800807162446396</v>
       </c>
       <c r="BD19" t="n">
-        <v>0.02551816773606724</v>
+        <v>0.02551816773606723</v>
       </c>
       <c r="BE19" t="n">
         <v>0.0004386830287683619</v>
@@ -10077,7 +10077,7 @@
         <v>0.0006174331599326156</v>
       </c>
       <c r="BG19" t="n">
-        <v>0.0008232866915907141</v>
+        <v>0.0008232866915907143</v>
       </c>
       <c r="BH19" t="n">
         <v>0.01477229576818847</v>
@@ -10089,16 +10089,16 @@
         <v>0.0001138877796868427</v>
       </c>
       <c r="BK19" t="n">
-        <v>0.007041476123928042</v>
+        <v>0.007041476123928045</v>
       </c>
       <c r="BL19" t="n">
         <v>8.572481697708279e-05</v>
       </c>
       <c r="BM19" t="n">
-        <v>0.02376213370278343</v>
+        <v>0.02376213370278344</v>
       </c>
       <c r="BN19" t="n">
-        <v>0.001256181450895547</v>
+        <v>0.001256181450895546</v>
       </c>
       <c r="BO19" t="n">
         <v>3.556478857712248e-05</v>
@@ -10116,7 +10116,7 @@
         <v>0.01721048914019958</v>
       </c>
       <c r="BT19" t="n">
-        <v>0.006198510844197337</v>
+        <v>0.00619851084419734</v>
       </c>
       <c r="BU19" t="n">
         <v>0.002624017943035063</v>
@@ -10125,7 +10125,7 @@
         <v>0.003060980414508927</v>
       </c>
       <c r="BW19" t="n">
-        <v>6.972303247226163e-06</v>
+        <v>6.972303247226166e-06</v>
       </c>
       <c r="BX19" t="n">
         <v>0.00219701899137024</v>
@@ -10137,7 +10137,7 @@
         <v>0.003198281833577727</v>
       </c>
       <c r="CA19" t="n">
-        <v>8.356084894294248e-05</v>
+        <v>8.356084894294251e-05</v>
       </c>
       <c r="CB19" t="n">
         <v>0.0003154503970550022</v>
@@ -10149,7 +10149,7 @@
         <v>0.0001736089479613229</v>
       </c>
       <c r="CE19" t="n">
-        <v>0.007016298094291307</v>
+        <v>0.007016298094291305</v>
       </c>
       <c r="CF19" t="n">
         <v>0.001368413499015502</v>
@@ -10203,7 +10203,7 @@
         <v>0.0002993265871351347</v>
       </c>
       <c r="CW19" t="n">
-        <v>0.000389150124026188</v>
+        <v>0.0003891501240261882</v>
       </c>
       <c r="CX19" t="n">
         <v>0.003452283542171334</v>
@@ -10233,13 +10233,13 @@
         <v>0.0003638613326867834</v>
       </c>
       <c r="DG19" t="n">
-        <v>0.004320271682123755</v>
+        <v>0.004320271682123752</v>
       </c>
       <c r="DH19" t="n">
         <v>0.0004185501942448721</v>
       </c>
       <c r="DI19" t="n">
-        <v>7.666997731471822e-05</v>
+        <v>7.666997731471819e-05</v>
       </c>
       <c r="DJ19" t="n">
         <v>4.225846497850852e-05</v>
@@ -10257,10 +10257,10 @@
         <v>3.241507591503502e-05</v>
       </c>
       <c r="DO19" t="n">
-        <v>0.0007871505645623628</v>
+        <v>0.0007871505645623626</v>
       </c>
       <c r="DP19" t="n">
-        <v>0.1531311298536745</v>
+        <v>0.1531311298536746</v>
       </c>
       <c r="DQ19" t="n">
         <v>4.962742212964996e-06</v>

</xml_diff>